<commit_message>
feat: Refactor agent 2
</commit_message>
<xml_diff>
--- a/llms_calls_accounting.xlsx
+++ b/llms_calls_accounting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\03_iastronauts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8B07905-F0BD-4527-B365-E4BAB9B0CA16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4781B0D5-CA31-4920-A0F1-B1808DC3E2AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{59B62FDA-1497-4401-82EC-1B2F7D702BCC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="28">
   <si>
     <t>Consumo Tokens CreditIQ</t>
   </si>
@@ -108,6 +108,21 @@
   </si>
   <si>
     <t>0.31</t>
+  </si>
+  <si>
+    <t>0.05</t>
+  </si>
+  <si>
+    <t>AFTER BIG REFACTOR</t>
+  </si>
+  <si>
+    <t>2026-05-27:13:12</t>
+  </si>
+  <si>
+    <t>2026-05-27:13:15</t>
+  </si>
+  <si>
+    <t>2026-05-27:13:47</t>
   </si>
 </sst>
 </file>
@@ -139,12 +154,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="11">
@@ -275,7 +296,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
@@ -283,6 +304,42 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -292,42 +349,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -662,287 +684,309 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B052F0D6-0E50-4E03-8DA0-D70F625DE32B}">
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.85546875" customWidth="1"/>
     <col min="2" max="2" width="13.28515625" customWidth="1"/>
     <col min="3" max="4" width="11.42578125" customWidth="1"/>
+    <col min="5" max="5" width="20.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="12"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="7"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="13" t="s">
+      <c r="B2" s="9"/>
+      <c r="C2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="14"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D2" s="9"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="19"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C3" s="15"/>
+      <c r="D3" s="16"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="16"/>
+      <c r="C4" s="11"/>
       <c r="D4" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="9"/>
+      <c r="C5" s="13"/>
       <c r="D5" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="9"/>
+      <c r="C6" s="13"/>
       <c r="D6" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="9"/>
+      <c r="C7" s="13"/>
       <c r="D7" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="9"/>
+      <c r="C8" s="13"/>
       <c r="D8" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="9"/>
+      <c r="C9" s="13"/>
       <c r="D9" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="9"/>
+      <c r="C10" s="13"/>
       <c r="D10" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="9"/>
+      <c r="C11" s="13"/>
       <c r="D11" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="9"/>
+      <c r="C12" s="13"/>
       <c r="D12" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="2"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="2"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="2"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="13"/>
+      <c r="D13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="20" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="13"/>
+      <c r="D14" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="13"/>
+      <c r="D15" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="9"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="13"/>
       <c r="D16" s="2"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="9"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="13"/>
       <c r="D17" s="2"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="9"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="13"/>
       <c r="D18" s="2"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="9"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="13"/>
       <c r="D19" s="2"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="9"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="13"/>
       <c r="D20" s="2"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="9"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="13"/>
       <c r="D21" s="2"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="9"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="13"/>
       <c r="D22" s="2"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="9"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="13"/>
       <c r="D23" s="2"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
-      <c r="B24" s="8"/>
-      <c r="C24" s="9"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="13"/>
       <c r="D24" s="2"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="9"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="13"/>
       <c r="D25" s="2"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="9"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="13"/>
       <c r="D26" s="2"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="8"/>
-      <c r="C27" s="9"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="13"/>
       <c r="D27" s="2"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="9"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="13"/>
       <c r="D28" s="2"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="9"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="13"/>
       <c r="D29" s="2"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
-      <c r="B30" s="5"/>
-      <c r="C30" s="6"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="18"/>
       <c r="D30" s="3"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
+      <c r="B31" s="19"/>
+      <c r="C31" s="19"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B32" s="7"/>
-      <c r="C32" s="7"/>
+      <c r="B32" s="19"/>
+      <c r="C32" s="19"/>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B33" s="7"/>
-      <c r="C33" s="7"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B34" s="7"/>
-      <c r="C34" s="7"/>
+      <c r="B34" s="19"/>
+      <c r="C34" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B18:C18"/>
@@ -951,22 +995,22 @@
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B7:C7"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B3:D3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Improved agent 1 and agent 2
</commit_message>
<xml_diff>
--- a/llms_calls_accounting.xlsx
+++ b/llms_calls_accounting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\03_iastronauts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4781B0D5-CA31-4920-A0F1-B1808DC3E2AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9BBD60F-4402-46D9-B596-96F810060EC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{59B62FDA-1497-4401-82EC-1B2F7D702BCC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="31">
   <si>
     <t>Consumo Tokens CreditIQ</t>
   </si>
@@ -123,6 +123,15 @@
   </si>
   <si>
     <t>2026-05-27:13:47</t>
+  </si>
+  <si>
+    <t>0.06</t>
+  </si>
+  <si>
+    <t>2026-05-27:22:02</t>
+  </si>
+  <si>
+    <t>2026-05-27:22:10</t>
   </si>
 </sst>
 </file>
@@ -304,6 +313,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -325,12 +350,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -340,16 +359,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -694,41 +703,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="7"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="13"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="8" t="s">
+      <c r="B2" s="15"/>
+      <c r="C2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="9"/>
+      <c r="D2" s="15"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="16"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="11"/>
+      <c r="C4" s="17"/>
       <c r="D4" s="4" t="s">
         <v>8</v>
       </c>
@@ -737,10 +746,10 @@
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="13"/>
+      <c r="C5" s="8"/>
       <c r="D5" s="2" t="s">
         <v>10</v>
       </c>
@@ -749,10 +758,10 @@
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="13"/>
+      <c r="C6" s="8"/>
       <c r="D6" s="2" t="s">
         <v>11</v>
       </c>
@@ -761,10 +770,10 @@
       <c r="A7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="13"/>
+      <c r="C7" s="8"/>
       <c r="D7" s="2" t="s">
         <v>10</v>
       </c>
@@ -773,10 +782,10 @@
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="13"/>
+      <c r="C8" s="8"/>
       <c r="D8" s="2" t="s">
         <v>16</v>
       </c>
@@ -785,10 +794,10 @@
       <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="13"/>
+      <c r="C9" s="8"/>
       <c r="D9" s="2" t="s">
         <v>10</v>
       </c>
@@ -797,10 +806,10 @@
       <c r="A10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="13"/>
+      <c r="C10" s="8"/>
       <c r="D10" s="2" t="s">
         <v>18</v>
       </c>
@@ -809,10 +818,10 @@
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="13"/>
+      <c r="C11" s="8"/>
       <c r="D11" s="2" t="s">
         <v>10</v>
       </c>
@@ -821,10 +830,10 @@
       <c r="A12" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="13"/>
+      <c r="C12" s="8"/>
       <c r="D12" s="2" t="s">
         <v>22</v>
       </c>
@@ -833,14 +842,14 @@
       <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="13"/>
+      <c r="C13" s="8"/>
       <c r="D13" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="20" t="s">
+      <c r="E13" s="5" t="s">
         <v>24</v>
       </c>
     </row>
@@ -848,10 +857,10 @@
       <c r="A14" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="13"/>
+      <c r="C14" s="8"/>
       <c r="D14" s="2" t="s">
         <v>23</v>
       </c>
@@ -860,133 +869,159 @@
       <c r="A15" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C15" s="13"/>
+      <c r="C15" s="8"/>
       <c r="D15" s="2" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="2"/>
+      <c r="A16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="8"/>
+      <c r="D16" s="2" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="2"/>
+      <c r="A17" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="8"/>
+      <c r="D17" s="2" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="13"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="8"/>
       <c r="D18" s="2"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="13"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="8"/>
       <c r="D19" s="2"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="13"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="8"/>
       <c r="D20" s="2"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="13"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="8"/>
       <c r="D21" s="2"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="13"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="8"/>
       <c r="D22" s="2"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="13"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="8"/>
       <c r="D23" s="2"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
-      <c r="B24" s="12"/>
-      <c r="C24" s="13"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="8"/>
       <c r="D24" s="2"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="13"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="8"/>
       <c r="D25" s="2"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="13"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="8"/>
       <c r="D26" s="2"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="13"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="8"/>
       <c r="D27" s="2"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
-      <c r="B28" s="12"/>
-      <c r="C28" s="13"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="8"/>
       <c r="D28" s="2"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="13"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="8"/>
       <c r="D29" s="2"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
-      <c r="B30" s="17"/>
-      <c r="C30" s="18"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="10"/>
       <c r="D30" s="3"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B31" s="19"/>
-      <c r="C31" s="19"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B32" s="19"/>
-      <c r="C32" s="19"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B34" s="19"/>
-      <c r="C34" s="19"/>
+      <c r="B34" s="6"/>
+      <c r="C34" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="35">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="B32:C32"/>
     <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B18:C18"/>
@@ -997,20 +1032,6 @@
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B3:D3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: Fixed cloud deploy, added secrets manager service and encapsule env vars
</commit_message>
<xml_diff>
--- a/llms_calls_accounting.xlsx
+++ b/llms_calls_accounting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\03_iastronauts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94887643-4730-4DF8-BE62-2813811C611A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE4EA7BB-C619-4150-86FC-7B7B9F083E25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{59B62FDA-1497-4401-82EC-1B2F7D702BCC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="40">
   <si>
     <t>Consumo Tokens CreditIQ</t>
   </si>
@@ -135,6 +135,30 @@
   </si>
   <si>
     <t>2026-05-30:01:47</t>
+  </si>
+  <si>
+    <t>P.ACCIONES</t>
+  </si>
+  <si>
+    <t>P.DINAMICO</t>
+  </si>
+  <si>
+    <t>2026-05-30:10:32</t>
+  </si>
+  <si>
+    <t>0.27</t>
+  </si>
+  <si>
+    <t>2026-05-30:10:37</t>
+  </si>
+  <si>
+    <t>0.7</t>
+  </si>
+  <si>
+    <t>2026-05-30:10:58</t>
+  </si>
+  <si>
+    <t>sonnet 4.6</t>
   </si>
 </sst>
 </file>
@@ -166,7 +190,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -179,8 +203,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -304,11 +334,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
@@ -317,6 +356,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -338,12 +392,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -353,15 +401,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -696,325 +739,553 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B052F0D6-0E50-4E03-8DA0-D70F625DE32B}">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.85546875" customWidth="1"/>
     <col min="2" max="2" width="13.28515625" customWidth="1"/>
     <col min="3" max="4" width="11.42578125" customWidth="1"/>
     <col min="5" max="5" width="20.140625" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" customWidth="1"/>
+    <col min="10" max="10" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="G1" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+    </row>
+    <row r="2" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="8"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="13"/>
+      <c r="G2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="13"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="9" t="s">
+      <c r="B3" s="15"/>
+      <c r="C3" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="10"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="D3" s="15"/>
+      <c r="G3" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" s="15"/>
+      <c r="I3" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="J3" s="15"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B4" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="17"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="C4" s="19"/>
+      <c r="D4" s="20"/>
+      <c r="G4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="I4" s="19"/>
+      <c r="J4" s="20"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B5" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="12"/>
-      <c r="D4" s="4" t="s">
+      <c r="C5" s="17"/>
+      <c r="D5" s="4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="G5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="I5" s="17"/>
+      <c r="J5" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="14"/>
-      <c r="D5" s="2" t="s">
+      <c r="C6" s="8"/>
+      <c r="D6" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="G6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="I6" s="8"/>
+      <c r="J6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K6" s="22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B7" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="14"/>
-      <c r="D6" s="2" t="s">
+      <c r="C7" s="8"/>
+      <c r="D7" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="G7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I7" s="8"/>
+      <c r="J7" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="K7" s="22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B8" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="14"/>
-      <c r="D7" s="2" t="s">
+      <c r="C8" s="8"/>
+      <c r="D8" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="G8" s="2"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="2"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="14"/>
-      <c r="D8" s="2" t="s">
+      <c r="C9" s="8"/>
+      <c r="D9" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="G9" s="2"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="2"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B10" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="2" t="s">
+      <c r="C10" s="8"/>
+      <c r="D10" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="G10" s="2"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="2"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B11" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="14"/>
-      <c r="D10" s="2" t="s">
+      <c r="C11" s="8"/>
+      <c r="D11" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="G11" s="2"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="2"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B12" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="14"/>
-      <c r="D11" s="2" t="s">
+      <c r="C12" s="8"/>
+      <c r="D12" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="G12" s="2"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="2"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B13" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="14"/>
-      <c r="D12" s="2" t="s">
+      <c r="C13" s="8"/>
+      <c r="D13" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="G13" s="2"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="2"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B14" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="14"/>
+      <c r="C14" s="8"/>
       <c r="D14" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E14" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G14" s="2"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="2"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" s="14"/>
+        <v>26</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="8"/>
       <c r="D15" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G15" s="2"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="2"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="8"/>
+      <c r="D16" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" s="2"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="2"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B17" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="14"/>
-      <c r="D16" s="2" t="s">
+      <c r="C17" s="8"/>
+      <c r="D17" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+      <c r="G17" s="2"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="2"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B18" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="14"/>
-      <c r="D17" s="2" t="s">
+      <c r="C18" s="8"/>
+      <c r="D18" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+      <c r="G18" s="2"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="2"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B19" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="2" t="s">
+      <c r="C19" s="8"/>
+      <c r="D19" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="2"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="2"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G19" s="2"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="2"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20" s="8"/>
+      <c r="D20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G20" s="2"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="2"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="14"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="8"/>
       <c r="D21" s="2"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G21" s="2"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="2"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="14"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="8"/>
       <c r="D22" s="2"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G22" s="2"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="2"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="13"/>
-      <c r="C23" s="14"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="8"/>
       <c r="D23" s="2"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G23" s="2"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="2"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="14"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="8"/>
       <c r="D24" s="2"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G24" s="2"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="2"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="14"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="8"/>
       <c r="D25" s="2"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G25" s="2"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="2"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="14"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="8"/>
       <c r="D26" s="2"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G26" s="2"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="2"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="13"/>
-      <c r="C27" s="14"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="8"/>
       <c r="D27" s="2"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G27" s="2"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="2"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="14"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="8"/>
       <c r="D28" s="2"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G28" s="2"/>
+      <c r="H28" s="7"/>
+      <c r="I28" s="8"/>
+      <c r="J28" s="2"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
-      <c r="B29" s="13"/>
-      <c r="C29" s="14"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="8"/>
       <c r="D29" s="2"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="3"/>
-      <c r="B30" s="19"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="3"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B32" s="18"/>
-      <c r="C32" s="18"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="7"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="2"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="2"/>
+      <c r="B30" s="7"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="8"/>
+      <c r="J30" s="2"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="3"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="9"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="3"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B33" s="18"/>
-      <c r="C33" s="18"/>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B34" s="18"/>
-      <c r="C34" s="18"/>
+      <c r="B34" s="6"/>
+      <c r="C34" s="6"/>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="35">
-    <mergeCell ref="B34:C34"/>
+  <mergeCells count="68">
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="G1:J1"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="G2:J2"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
     <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B18:C18"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="B32:C32"/>
     <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B34:C34"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B21:C21"/>
@@ -1023,24 +1294,6 @@
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B3:D3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Improving GUI. Added animations, modified cards. Improve Risk Analyzer
</commit_message>
<xml_diff>
--- a/llms_calls_accounting.xlsx
+++ b/llms_calls_accounting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\03_iastronauts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE4EA7BB-C619-4150-86FC-7B7B9F083E25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8A94FAB-6BBC-4233-A333-5A3D2841226C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{59B62FDA-1497-4401-82EC-1B2F7D702BCC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="43">
   <si>
     <t>Consumo Tokens CreditIQ</t>
   </si>
@@ -159,13 +159,22 @@
   </si>
   <si>
     <t>sonnet 4.6</t>
+  </si>
+  <si>
+    <t>2026-05-30:13:34</t>
+  </si>
+  <si>
+    <t>RiskAnalyzer</t>
+  </si>
+  <si>
+    <t>haiku 4.6</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -185,6 +194,12 @@
       <b/>
       <sz val="14"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -347,7 +362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
@@ -356,55 +371,56 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -739,545 +755,546 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B052F0D6-0E50-4E03-8DA0-D70F625DE32B}">
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.85546875" customWidth="1"/>
     <col min="2" max="2" width="13.28515625" customWidth="1"/>
     <col min="3" max="4" width="11.42578125" customWidth="1"/>
     <col min="5" max="5" width="20.140625" customWidth="1"/>
-    <col min="7" max="7" width="15.42578125" customWidth="1"/>
-    <col min="9" max="9" width="15.85546875" customWidth="1"/>
-    <col min="10" max="10" width="17.85546875" customWidth="1"/>
+    <col min="9" max="9" width="15.42578125" customWidth="1"/>
+    <col min="11" max="11" width="15.85546875" customWidth="1"/>
+    <col min="12" max="12" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="G1" s="21" t="s">
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="I1" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-    </row>
-    <row r="2" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+    </row>
+    <row r="2" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="13"/>
-      <c r="G2" s="11" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="14"/>
+      <c r="I2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
       <c r="J2" s="13"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="K2" s="13"/>
+      <c r="L2" s="14"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="15"/>
-      <c r="C3" s="14" t="s">
+      <c r="B3" s="16"/>
+      <c r="C3" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="15"/>
-      <c r="G3" s="14" t="s">
+      <c r="D3" s="16"/>
+      <c r="I3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="H3" s="15"/>
-      <c r="I3" s="14" t="s">
+      <c r="J3" s="16"/>
+      <c r="K3" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="15"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L3" s="16"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="20"/>
-      <c r="G4" s="1" t="s">
+      <c r="C4" s="18"/>
+      <c r="D4" s="19"/>
+      <c r="I4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="18" t="s">
+      <c r="J4" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="19"/>
-      <c r="J4" s="20"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K4" s="18"/>
+      <c r="L4" s="19"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="17"/>
+      <c r="C5" s="21"/>
       <c r="D5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="I5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="16" t="s">
+      <c r="J5" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="I5" s="17"/>
-      <c r="J5" s="4" t="s">
+      <c r="K5" s="21"/>
+      <c r="L5" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="8"/>
+      <c r="C6" s="11"/>
       <c r="D6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="E6" t="s">
+        <v>42</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="J6" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="8"/>
-      <c r="J6" s="2" t="s">
+      <c r="K6" s="11"/>
+      <c r="L6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="K6" s="22" t="s">
+      <c r="M6" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="8"/>
+      <c r="C7" s="11"/>
       <c r="D7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="E7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="J7" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="I7" s="8"/>
-      <c r="J7" s="2" t="s">
+      <c r="K7" s="11"/>
+      <c r="L7" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="K7" s="22" t="s">
+      <c r="M7" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="8"/>
+      <c r="C8" s="11"/>
       <c r="D8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="2"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="2"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
+        <v>42</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="K8" s="11"/>
+      <c r="L8" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="8"/>
+      <c r="C9" s="11"/>
       <c r="D9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="2"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="2"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E9" t="s">
+        <v>42</v>
+      </c>
+      <c r="I9" s="2"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="2"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="8"/>
+      <c r="C10" s="11"/>
       <c r="D10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G10" s="2"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="2"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E10" t="s">
+        <v>42</v>
+      </c>
+      <c r="I10" s="2"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="2"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="8"/>
+      <c r="C11" s="11"/>
       <c r="D11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G11" s="2"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="2"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E11" t="s">
+        <v>42</v>
+      </c>
+      <c r="I11" s="2"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="2"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="8"/>
+      <c r="C12" s="11"/>
       <c r="D12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G12" s="2"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="2"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E12" t="s">
+        <v>42</v>
+      </c>
+      <c r="I12" s="2"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="2"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="8"/>
+      <c r="C13" s="11"/>
       <c r="D13" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G13" s="2"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="2"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E13" t="s">
+        <v>42</v>
+      </c>
+      <c r="I13" s="2"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="2"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="8"/>
+      <c r="C14" s="11"/>
       <c r="D14" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" t="s">
+        <v>42</v>
+      </c>
+      <c r="F14" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="G14" s="2"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="2"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G14" s="5"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="2"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="8"/>
+      <c r="C15" s="11"/>
       <c r="D15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G15" s="2"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="2"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E15" t="s">
+        <v>42</v>
+      </c>
+      <c r="I15" s="2"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="2"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="8"/>
+      <c r="C16" s="11"/>
       <c r="D16" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G16" s="2"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="2"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E16" t="s">
+        <v>42</v>
+      </c>
+      <c r="I16" s="2"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="2"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C17" s="8"/>
+      <c r="C17" s="11"/>
       <c r="D17" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="G17" s="2"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="2"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E17" t="s">
+        <v>42</v>
+      </c>
+      <c r="I17" s="2"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="2"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="8"/>
+      <c r="C18" s="11"/>
       <c r="D18" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G18" s="2"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="2"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E18" t="s">
+        <v>42</v>
+      </c>
+      <c r="I18" s="2"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="2"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="8"/>
+      <c r="C19" s="11"/>
       <c r="D19" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="G19" s="2"/>
-      <c r="H19" s="7"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="2"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E19" t="s">
+        <v>42</v>
+      </c>
+      <c r="I19" s="2"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="2"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C20" s="8"/>
+      <c r="C20" s="11"/>
       <c r="D20" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G20" s="2"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="2"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E20" t="s">
+        <v>42</v>
+      </c>
+      <c r="I20" s="2"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="2"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="8"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="11"/>
       <c r="D21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="2"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I21" s="2"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="2"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="8"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="11"/>
       <c r="D22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="7"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="2"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I22" s="2"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="11"/>
+      <c r="L22" s="2"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="8"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="11"/>
       <c r="D23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="2"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I23" s="2"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="11"/>
+      <c r="L23" s="2"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
-      <c r="B24" s="7"/>
-      <c r="C24" s="8"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="11"/>
       <c r="D24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="2"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I24" s="2"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="11"/>
+      <c r="L24" s="2"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="7"/>
-      <c r="C25" s="8"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="11"/>
       <c r="D25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="2"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I25" s="2"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="11"/>
+      <c r="L25" s="2"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
-      <c r="B26" s="7"/>
-      <c r="C26" s="8"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="11"/>
       <c r="D26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="2"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I26" s="2"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="11"/>
+      <c r="L26" s="2"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="7"/>
-      <c r="C27" s="8"/>
+      <c r="B27" s="10"/>
+      <c r="C27" s="11"/>
       <c r="D27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="8"/>
-      <c r="J27" s="2"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I27" s="2"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="11"/>
+      <c r="L27" s="2"/>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
-      <c r="B28" s="7"/>
-      <c r="C28" s="8"/>
+      <c r="B28" s="10"/>
+      <c r="C28" s="11"/>
       <c r="D28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="8"/>
-      <c r="J28" s="2"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I28" s="2"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="11"/>
+      <c r="L28" s="2"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
-      <c r="B29" s="7"/>
-      <c r="C29" s="8"/>
+      <c r="B29" s="10"/>
+      <c r="C29" s="11"/>
       <c r="D29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="7"/>
-      <c r="I29" s="8"/>
-      <c r="J29" s="2"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I29" s="2"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="11"/>
+      <c r="L29" s="2"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
-      <c r="B30" s="7"/>
-      <c r="C30" s="8"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="11"/>
       <c r="D30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="7"/>
-      <c r="I30" s="8"/>
-      <c r="J30" s="2"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I30" s="2"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="11"/>
+      <c r="L30" s="2"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
-      <c r="B31" s="9"/>
-      <c r="C31" s="10"/>
+      <c r="B31" s="7"/>
+      <c r="C31" s="8"/>
       <c r="D31" s="3"/>
-      <c r="G31" s="3"/>
-      <c r="H31" s="9"/>
-      <c r="I31" s="10"/>
-      <c r="J31" s="3"/>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B32" s="6"/>
-      <c r="C32" s="6"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="7"/>
+      <c r="K31" s="8"/>
+      <c r="L31" s="3"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B32" s="22"/>
+      <c r="C32" s="22"/>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B33" s="6"/>
-      <c r="C33" s="6"/>
+      <c r="B33" s="22"/>
+      <c r="C33" s="22"/>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B34" s="6"/>
-      <c r="C34" s="6"/>
+      <c r="B34" s="22"/>
+      <c r="C34" s="22"/>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B35" s="6"/>
-      <c r="C35" s="6"/>
+      <c r="B35" s="22"/>
+      <c r="C35" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="68">
-    <mergeCell ref="H31:I31"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="G1:J1"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="H28:I28"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="G2:J2"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B31:C31"/>
@@ -1294,7 +1311,60 @@
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="I1:L1"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
   </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: Fixed cards position
</commit_message>
<xml_diff>
--- a/llms_calls_accounting.xlsx
+++ b/llms_calls_accounting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\03_iastronauts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8A94FAB-6BBC-4233-A333-5A3D2841226C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{313DB9A3-50C5-4107-ADB7-0138874484FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{59B62FDA-1497-4401-82EC-1B2F7D702BCC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="47">
   <si>
     <t>Consumo Tokens CreditIQ</t>
   </si>
@@ -168,6 +168,18 @@
   </si>
   <si>
     <t>haiku 4.6</t>
+  </si>
+  <si>
+    <t>2026-05-30:16:02</t>
+  </si>
+  <si>
+    <t>0.07</t>
+  </si>
+  <si>
+    <t>2026-05-30:16:05</t>
+  </si>
+  <si>
+    <t>0.01</t>
   </si>
 </sst>
 </file>
@@ -362,7 +374,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
@@ -372,21 +384,27 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -411,16 +429,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -755,7 +766,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B052F0D6-0E50-4E03-8DA0-D70F625DE32B}">
-  <dimension ref="A1:M35"/>
+  <dimension ref="A1:S35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.85546875" customWidth="1"/>
@@ -765,102 +776,142 @@
     <col min="9" max="9" width="15.42578125" customWidth="1"/>
     <col min="11" max="11" width="15.85546875" customWidth="1"/>
     <col min="12" max="12" width="17.85546875" customWidth="1"/>
+    <col min="16" max="16" width="17.140625" customWidth="1"/>
+    <col min="18" max="18" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="I1" s="9" t="s">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="I1" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-    </row>
-    <row r="2" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="P1" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13"/>
+      <c r="S1" s="13"/>
+    </row>
+    <row r="2" spans="1:19" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A2" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="14"/>
-      <c r="I2" s="12" t="s">
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="16"/>
+      <c r="I2" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="J2" s="13"/>
-      <c r="K2" s="13"/>
-      <c r="L2" s="14"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+      <c r="L2" s="16"/>
+      <c r="P2" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="15"/>
+      <c r="R2" s="15"/>
+      <c r="S2" s="16"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="15" t="s">
+      <c r="B3" s="18"/>
+      <c r="C3" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="16"/>
-      <c r="I3" s="15" t="s">
+      <c r="D3" s="18"/>
+      <c r="I3" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="16"/>
-      <c r="K3" s="15" t="s">
+      <c r="J3" s="18"/>
+      <c r="K3" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="16"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="L3" s="18"/>
+      <c r="P3" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="18"/>
+      <c r="R3" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="S3" s="18"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="18"/>
-      <c r="D4" s="19"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="21"/>
       <c r="I4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="17" t="s">
+      <c r="J4" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="18"/>
-      <c r="L4" s="19"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K4" s="20"/>
+      <c r="L4" s="21"/>
+      <c r="P4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="R4" s="20"/>
+      <c r="S4" s="21"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="21"/>
+      <c r="C5" s="12"/>
       <c r="D5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="20" t="s">
+      <c r="J5" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="K5" s="21"/>
+      <c r="K5" s="12"/>
       <c r="L5" s="4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="R5" s="12"/>
+      <c r="S5" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="11"/>
+      <c r="C6" s="8"/>
       <c r="D6" s="2" t="s">
         <v>10</v>
       </c>
@@ -870,25 +921,35 @@
       <c r="I6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J6" s="10" t="s">
+      <c r="J6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="K6" s="11"/>
+      <c r="K6" s="8"/>
       <c r="L6" s="2" t="s">
         <v>35</v>
       </c>
       <c r="M6" s="6" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q6" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="R6" s="8"/>
+      <c r="S6" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="11"/>
+      <c r="C7" s="8"/>
       <c r="D7" s="2" t="s">
         <v>11</v>
       </c>
@@ -898,25 +959,35 @@
       <c r="I7" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="J7" s="10" t="s">
+      <c r="J7" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="K7" s="11"/>
+      <c r="K7" s="8"/>
       <c r="L7" s="2" t="s">
         <v>37</v>
       </c>
       <c r="M7" s="6" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="R7" s="8"/>
+      <c r="S7" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="11"/>
+      <c r="C8" s="8"/>
       <c r="D8" s="2" t="s">
         <v>10</v>
       </c>
@@ -926,22 +997,32 @@
       <c r="I8" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="J8" s="10" t="s">
+      <c r="J8" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="K8" s="11"/>
+      <c r="K8" s="8"/>
       <c r="L8" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P8" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q8" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="R8" s="8"/>
+      <c r="S8" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="11"/>
+      <c r="C9" s="8"/>
       <c r="D9" s="2" t="s">
         <v>16</v>
       </c>
@@ -949,18 +1030,22 @@
         <v>42</v>
       </c>
       <c r="I9" s="2"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="11"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="8"/>
       <c r="L9" s="2"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P9" s="2"/>
+      <c r="Q9" s="7"/>
+      <c r="R9" s="8"/>
+      <c r="S9" s="2"/>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="11"/>
+      <c r="C10" s="8"/>
       <c r="D10" s="2" t="s">
         <v>10</v>
       </c>
@@ -968,18 +1053,22 @@
         <v>42</v>
       </c>
       <c r="I10" s="2"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="11"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="8"/>
       <c r="L10" s="2"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P10" s="2"/>
+      <c r="Q10" s="7"/>
+      <c r="R10" s="8"/>
+      <c r="S10" s="2"/>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="11"/>
+      <c r="C11" s="8"/>
       <c r="D11" s="2" t="s">
         <v>18</v>
       </c>
@@ -987,18 +1076,22 @@
         <v>42</v>
       </c>
       <c r="I11" s="2"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="11"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="8"/>
       <c r="L11" s="2"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P11" s="2"/>
+      <c r="Q11" s="7"/>
+      <c r="R11" s="8"/>
+      <c r="S11" s="2"/>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="11"/>
+      <c r="C12" s="8"/>
       <c r="D12" s="2" t="s">
         <v>10</v>
       </c>
@@ -1006,18 +1099,22 @@
         <v>42</v>
       </c>
       <c r="I12" s="2"/>
-      <c r="J12" s="10"/>
-      <c r="K12" s="11"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="8"/>
       <c r="L12" s="2"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P12" s="2"/>
+      <c r="Q12" s="7"/>
+      <c r="R12" s="8"/>
+      <c r="S12" s="2"/>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="11"/>
+      <c r="C13" s="8"/>
       <c r="D13" s="2" t="s">
         <v>22</v>
       </c>
@@ -1025,18 +1122,22 @@
         <v>42</v>
       </c>
       <c r="I13" s="2"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="11"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="8"/>
       <c r="L13" s="2"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P13" s="2"/>
+      <c r="Q13" s="7"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="2"/>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="11"/>
+      <c r="C14" s="8"/>
       <c r="D14" s="2" t="s">
         <v>23</v>
       </c>
@@ -1047,20 +1148,23 @@
         <v>24</v>
       </c>
       <c r="G14" s="5"/>
-      <c r="H14" s="23"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="11"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="8"/>
       <c r="L14" s="2"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P14" s="2"/>
+      <c r="Q14" s="7"/>
+      <c r="R14" s="8"/>
+      <c r="S14" s="2"/>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="11"/>
+      <c r="C15" s="8"/>
       <c r="D15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1068,18 +1172,22 @@
         <v>42</v>
       </c>
       <c r="I15" s="2"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="11"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="8"/>
       <c r="L15" s="2"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P15" s="2"/>
+      <c r="Q15" s="7"/>
+      <c r="R15" s="8"/>
+      <c r="S15" s="2"/>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="11"/>
+      <c r="C16" s="8"/>
       <c r="D16" s="2" t="s">
         <v>23</v>
       </c>
@@ -1087,18 +1195,22 @@
         <v>42</v>
       </c>
       <c r="I16" s="2"/>
-      <c r="J16" s="10"/>
-      <c r="K16" s="11"/>
+      <c r="J16" s="7"/>
+      <c r="K16" s="8"/>
       <c r="L16" s="2"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="P16" s="2"/>
+      <c r="Q16" s="7"/>
+      <c r="R16" s="8"/>
+      <c r="S16" s="2"/>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C17" s="11"/>
+      <c r="C17" s="8"/>
       <c r="D17" s="2" t="s">
         <v>28</v>
       </c>
@@ -1106,18 +1218,22 @@
         <v>42</v>
       </c>
       <c r="I17" s="2"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="11"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="8"/>
       <c r="L17" s="2"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="P17" s="2"/>
+      <c r="Q17" s="7"/>
+      <c r="R17" s="8"/>
+      <c r="S17" s="2"/>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="11"/>
+      <c r="C18" s="8"/>
       <c r="D18" s="2" t="s">
         <v>23</v>
       </c>
@@ -1125,18 +1241,22 @@
         <v>42</v>
       </c>
       <c r="I18" s="2"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="11"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="8"/>
       <c r="L18" s="2"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="P18" s="2"/>
+      <c r="Q18" s="7"/>
+      <c r="R18" s="8"/>
+      <c r="S18" s="2"/>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="11"/>
+      <c r="C19" s="8"/>
       <c r="D19" s="2" t="s">
         <v>28</v>
       </c>
@@ -1144,18 +1264,22 @@
         <v>42</v>
       </c>
       <c r="I19" s="2"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="11"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="8"/>
       <c r="L19" s="2"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="P19" s="2"/>
+      <c r="Q19" s="7"/>
+      <c r="R19" s="8"/>
+      <c r="S19" s="2"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C20" s="11"/>
+      <c r="C20" s="8"/>
       <c r="D20" s="2" t="s">
         <v>35</v>
       </c>
@@ -1163,121 +1287,169 @@
         <v>42</v>
       </c>
       <c r="I20" s="2"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="11"/>
+      <c r="J20" s="7"/>
+      <c r="K20" s="8"/>
       <c r="L20" s="2"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="P20" s="2"/>
+      <c r="Q20" s="7"/>
+      <c r="R20" s="8"/>
+      <c r="S20" s="2"/>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="11"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="8"/>
       <c r="D21" s="2"/>
       <c r="I21" s="2"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="11"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="8"/>
       <c r="L21" s="2"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="P21" s="2"/>
+      <c r="Q21" s="7"/>
+      <c r="R21" s="8"/>
+      <c r="S21" s="2"/>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="11"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="8"/>
       <c r="D22" s="2"/>
       <c r="I22" s="2"/>
-      <c r="J22" s="10"/>
-      <c r="K22" s="11"/>
+      <c r="J22" s="7"/>
+      <c r="K22" s="8"/>
       <c r="L22" s="2"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="P22" s="2"/>
+      <c r="Q22" s="7"/>
+      <c r="R22" s="8"/>
+      <c r="S22" s="2"/>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="11"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="8"/>
       <c r="D23" s="2"/>
       <c r="I23" s="2"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="11"/>
+      <c r="J23" s="7"/>
+      <c r="K23" s="8"/>
       <c r="L23" s="2"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="P23" s="2"/>
+      <c r="Q23" s="7"/>
+      <c r="R23" s="8"/>
+      <c r="S23" s="2"/>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="11"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="8"/>
       <c r="D24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="10"/>
-      <c r="K24" s="11"/>
+      <c r="J24" s="7"/>
+      <c r="K24" s="8"/>
       <c r="L24" s="2"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="P24" s="2"/>
+      <c r="Q24" s="7"/>
+      <c r="R24" s="8"/>
+      <c r="S24" s="2"/>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="11"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="8"/>
       <c r="D25" s="2"/>
       <c r="I25" s="2"/>
-      <c r="J25" s="10"/>
-      <c r="K25" s="11"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="8"/>
       <c r="L25" s="2"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="P25" s="2"/>
+      <c r="Q25" s="7"/>
+      <c r="R25" s="8"/>
+      <c r="S25" s="2"/>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="11"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="8"/>
       <c r="D26" s="2"/>
       <c r="I26" s="2"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="11"/>
+      <c r="J26" s="7"/>
+      <c r="K26" s="8"/>
       <c r="L26" s="2"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="P26" s="2"/>
+      <c r="Q26" s="7"/>
+      <c r="R26" s="8"/>
+      <c r="S26" s="2"/>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="11"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="8"/>
       <c r="D27" s="2"/>
       <c r="I27" s="2"/>
-      <c r="J27" s="10"/>
-      <c r="K27" s="11"/>
+      <c r="J27" s="7"/>
+      <c r="K27" s="8"/>
       <c r="L27" s="2"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="P27" s="2"/>
+      <c r="Q27" s="7"/>
+      <c r="R27" s="8"/>
+      <c r="S27" s="2"/>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="11"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="8"/>
       <c r="D28" s="2"/>
       <c r="I28" s="2"/>
-      <c r="J28" s="10"/>
-      <c r="K28" s="11"/>
+      <c r="J28" s="7"/>
+      <c r="K28" s="8"/>
       <c r="L28" s="2"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="P28" s="2"/>
+      <c r="Q28" s="7"/>
+      <c r="R28" s="8"/>
+      <c r="S28" s="2"/>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="11"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="8"/>
       <c r="D29" s="2"/>
       <c r="I29" s="2"/>
-      <c r="J29" s="10"/>
-      <c r="K29" s="11"/>
+      <c r="J29" s="7"/>
+      <c r="K29" s="8"/>
       <c r="L29" s="2"/>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="P29" s="2"/>
+      <c r="Q29" s="7"/>
+      <c r="R29" s="8"/>
+      <c r="S29" s="2"/>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="11"/>
+      <c r="B30" s="7"/>
+      <c r="C30" s="8"/>
       <c r="D30" s="2"/>
       <c r="I30" s="2"/>
-      <c r="J30" s="10"/>
-      <c r="K30" s="11"/>
+      <c r="J30" s="7"/>
+      <c r="K30" s="8"/>
       <c r="L30" s="2"/>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="P30" s="2"/>
+      <c r="Q30" s="7"/>
+      <c r="R30" s="8"/>
+      <c r="S30" s="2"/>
+    </row>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
-      <c r="B31" s="7"/>
-      <c r="C31" s="8"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="10"/>
       <c r="D31" s="3"/>
       <c r="I31" s="3"/>
-      <c r="J31" s="7"/>
-      <c r="K31" s="8"/>
+      <c r="J31" s="9"/>
+      <c r="K31" s="10"/>
       <c r="L31" s="3"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="P31" s="3"/>
+      <c r="Q31" s="9"/>
+      <c r="R31" s="10"/>
+      <c r="S31" s="3"/>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B32" s="22"/>
       <c r="C32" s="22"/>
     </row>
@@ -1294,7 +1466,7 @@
       <c r="C35" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="68">
+  <mergeCells count="100">
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B31:C31"/>
@@ -1363,6 +1535,38 @@
     <mergeCell ref="J16:K16"/>
     <mergeCell ref="J17:K17"/>
     <mergeCell ref="J18:K18"/>
+    <mergeCell ref="P1:S1"/>
+    <mergeCell ref="P2:S2"/>
+    <mergeCell ref="P3:Q3"/>
+    <mergeCell ref="R3:S3"/>
+    <mergeCell ref="Q4:S4"/>
+    <mergeCell ref="Q5:R5"/>
+    <mergeCell ref="Q6:R6"/>
+    <mergeCell ref="Q7:R7"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="Q9:R9"/>
+    <mergeCell ref="Q10:R10"/>
+    <mergeCell ref="Q11:R11"/>
+    <mergeCell ref="Q12:R12"/>
+    <mergeCell ref="Q13:R13"/>
+    <mergeCell ref="Q14:R14"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="Q16:R16"/>
+    <mergeCell ref="Q17:R17"/>
+    <mergeCell ref="Q18:R18"/>
+    <mergeCell ref="Q19:R19"/>
+    <mergeCell ref="Q20:R20"/>
+    <mergeCell ref="Q21:R21"/>
+    <mergeCell ref="Q22:R22"/>
+    <mergeCell ref="Q23:R23"/>
+    <mergeCell ref="Q24:R24"/>
+    <mergeCell ref="Q30:R30"/>
+    <mergeCell ref="Q31:R31"/>
+    <mergeCell ref="Q25:R25"/>
+    <mergeCell ref="Q26:R26"/>
+    <mergeCell ref="Q27:R27"/>
+    <mergeCell ref="Q28:R28"/>
+    <mergeCell ref="Q29:R29"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: Modified news viewing and markets view
</commit_message>
<xml_diff>
--- a/llms_calls_accounting.xlsx
+++ b/llms_calls_accounting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\03_iastronauts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{313DB9A3-50C5-4107-ADB7-0138874484FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8CC3B22-24CB-45DF-8265-1C0E63A78934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{59B62FDA-1497-4401-82EC-1B2F7D702BCC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="49">
   <si>
     <t>Consumo Tokens CreditIQ</t>
   </si>
@@ -180,6 +180,12 @@
   </si>
   <si>
     <t>0.01</t>
+  </si>
+  <si>
+    <t>2026-05-31:13:34</t>
+  </si>
+  <si>
+    <t>2026-05-31:13:35</t>
   </si>
 </sst>
 </file>
@@ -374,7 +380,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
@@ -384,6 +390,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -396,41 +405,45 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -766,7 +779,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B052F0D6-0E50-4E03-8DA0-D70F625DE32B}">
-  <dimension ref="A1:S35"/>
+  <dimension ref="A1:T35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.85546875" customWidth="1"/>
@@ -780,73 +793,73 @@
     <col min="18" max="18" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A1" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="I1" s="13" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="I1" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="P1" s="13" t="s">
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="P1" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="Q1" s="13"/>
-      <c r="R1" s="13"/>
-      <c r="S1" s="13"/>
-    </row>
-    <row r="2" spans="1:19" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
+      <c r="Q1" s="22"/>
+      <c r="R1" s="22"/>
+      <c r="S1" s="22"/>
+    </row>
+    <row r="2" spans="1:20" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="16"/>
-      <c r="I2" s="14" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="14"/>
+      <c r="I2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="16"/>
-      <c r="P2" s="14" t="s">
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="14"/>
+      <c r="P2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="Q2" s="15"/>
-      <c r="R2" s="15"/>
-      <c r="S2" s="16"/>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="14"/>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="17" t="s">
+      <c r="B3" s="16"/>
+      <c r="C3" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="18"/>
-      <c r="I3" s="17" t="s">
+      <c r="D3" s="16"/>
+      <c r="I3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="18"/>
-      <c r="K3" s="17" t="s">
+      <c r="J3" s="16"/>
+      <c r="K3" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="18"/>
-      <c r="P3" s="17" t="s">
+      <c r="L3" s="16"/>
+      <c r="P3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="Q3" s="18"/>
-      <c r="R3" s="17" t="s">
+      <c r="Q3" s="16"/>
+      <c r="R3" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="S3" s="18"/>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S3" s="16"/>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -872,46 +885,46 @@
       <c r="R4" s="20"/>
       <c r="S4" s="21"/>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="12"/>
+      <c r="C5" s="18"/>
       <c r="D5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="11" t="s">
+      <c r="J5" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="K5" s="12"/>
+      <c r="K5" s="18"/>
       <c r="L5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="P5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="Q5" s="11" t="s">
+      <c r="Q5" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="R5" s="12"/>
+      <c r="R5" s="18"/>
       <c r="S5" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="8"/>
+      <c r="C6" s="9"/>
       <c r="D6" s="2" t="s">
         <v>10</v>
       </c>
@@ -921,10 +934,10 @@
       <c r="I6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="J6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="K6" s="8"/>
+      <c r="K6" s="9"/>
       <c r="L6" s="2" t="s">
         <v>35</v>
       </c>
@@ -934,22 +947,25 @@
       <c r="P6" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="Q6" s="7" t="s">
+      <c r="Q6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="R6" s="8"/>
+      <c r="R6" s="9"/>
       <c r="S6" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="8"/>
+      <c r="C7" s="9"/>
       <c r="D7" s="2" t="s">
         <v>11</v>
       </c>
@@ -959,10 +975,10 @@
       <c r="I7" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="J7" s="7" t="s">
+      <c r="J7" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="K7" s="8"/>
+      <c r="K7" s="9"/>
       <c r="L7" s="2" t="s">
         <v>37</v>
       </c>
@@ -972,22 +988,25 @@
       <c r="P7" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="Q7" s="7" t="s">
+      <c r="Q7" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="R7" s="8"/>
+      <c r="R7" s="9"/>
       <c r="S7" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="8"/>
+      <c r="C8" s="9"/>
       <c r="D8" s="2" t="s">
         <v>10</v>
       </c>
@@ -997,101 +1016,134 @@
       <c r="I8" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="J8" s="7" t="s">
+      <c r="J8" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="K8" s="8"/>
+      <c r="K8" s="9"/>
       <c r="L8" s="2" t="s">
         <v>23</v>
       </c>
+      <c r="M8" t="s">
+        <v>42</v>
+      </c>
       <c r="P8" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="Q8" s="7" t="s">
+      <c r="Q8" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="R8" s="8"/>
+      <c r="R8" s="9"/>
       <c r="S8" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="8"/>
+      <c r="C9" s="9"/>
       <c r="D9" s="2" t="s">
         <v>16</v>
       </c>
       <c r="E9" t="s">
         <v>42</v>
       </c>
-      <c r="I9" s="2"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="8"/>
-      <c r="L9" s="2"/>
+      <c r="I9" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="K9" s="9"/>
+      <c r="L9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M9" t="s">
+        <v>42</v>
+      </c>
       <c r="P9" s="2"/>
-      <c r="Q9" s="7"/>
-      <c r="R9" s="8"/>
+      <c r="Q9" s="8"/>
+      <c r="R9" s="9"/>
       <c r="S9" s="2"/>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="8"/>
+      <c r="C10" s="9"/>
       <c r="D10" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E10" t="s">
         <v>42</v>
       </c>
-      <c r="I10" s="2"/>
-      <c r="J10" s="7"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="2"/>
+      <c r="I10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K10" s="9"/>
+      <c r="L10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M10" t="s">
+        <v>42</v>
+      </c>
       <c r="P10" s="2"/>
-      <c r="Q10" s="7"/>
-      <c r="R10" s="8"/>
+      <c r="Q10" s="8"/>
+      <c r="R10" s="9"/>
       <c r="S10" s="2"/>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="8"/>
+      <c r="C11" s="9"/>
       <c r="D11" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E11" t="s">
         <v>42</v>
       </c>
-      <c r="I11" s="2"/>
-      <c r="J11" s="7"/>
-      <c r="K11" s="8"/>
-      <c r="L11" s="2"/>
+      <c r="I11" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="K11" s="9"/>
+      <c r="L11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="M11" t="s">
+        <v>42</v>
+      </c>
       <c r="P11" s="2"/>
-      <c r="Q11" s="7"/>
-      <c r="R11" s="8"/>
+      <c r="Q11" s="8"/>
+      <c r="R11" s="9"/>
       <c r="S11" s="2"/>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="8"/>
+      <c r="C12" s="9"/>
       <c r="D12" s="2" t="s">
         <v>10</v>
       </c>
@@ -1099,22 +1151,22 @@
         <v>42</v>
       </c>
       <c r="I12" s="2"/>
-      <c r="J12" s="7"/>
-      <c r="K12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="9"/>
       <c r="L12" s="2"/>
       <c r="P12" s="2"/>
-      <c r="Q12" s="7"/>
-      <c r="R12" s="8"/>
+      <c r="Q12" s="8"/>
+      <c r="R12" s="9"/>
       <c r="S12" s="2"/>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="8"/>
+      <c r="C13" s="9"/>
       <c r="D13" s="2" t="s">
         <v>22</v>
       </c>
@@ -1122,26 +1174,26 @@
         <v>42</v>
       </c>
       <c r="I13" s="2"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="9"/>
       <c r="L13" s="2"/>
       <c r="P13" s="2"/>
-      <c r="Q13" s="7"/>
-      <c r="R13" s="8"/>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="9"/>
       <c r="S13" s="2"/>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A14" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="8"/>
-      <c r="D14" s="2" t="s">
+      <c r="C14" s="25"/>
+      <c r="D14" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="5" t="s">
         <v>42</v>
       </c>
       <c r="F14" s="5" t="s">
@@ -1149,22 +1201,22 @@
       </c>
       <c r="G14" s="5"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="7"/>
-      <c r="K14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="9"/>
       <c r="L14" s="2"/>
       <c r="P14" s="2"/>
-      <c r="Q14" s="7"/>
-      <c r="R14" s="8"/>
+      <c r="Q14" s="8"/>
+      <c r="R14" s="9"/>
       <c r="S14" s="2"/>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="8"/>
+      <c r="C15" s="9"/>
       <c r="D15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1172,22 +1224,22 @@
         <v>42</v>
       </c>
       <c r="I15" s="2"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="9"/>
       <c r="L15" s="2"/>
       <c r="P15" s="2"/>
-      <c r="Q15" s="7"/>
-      <c r="R15" s="8"/>
+      <c r="Q15" s="8"/>
+      <c r="R15" s="9"/>
       <c r="S15" s="2"/>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="8"/>
+      <c r="C16" s="9"/>
       <c r="D16" s="2" t="s">
         <v>23</v>
       </c>
@@ -1195,22 +1247,22 @@
         <v>42</v>
       </c>
       <c r="I16" s="2"/>
-      <c r="J16" s="7"/>
-      <c r="K16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="9"/>
       <c r="L16" s="2"/>
       <c r="P16" s="2"/>
-      <c r="Q16" s="7"/>
-      <c r="R16" s="8"/>
+      <c r="Q16" s="8"/>
+      <c r="R16" s="9"/>
       <c r="S16" s="2"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C17" s="8"/>
+      <c r="C17" s="9"/>
       <c r="D17" s="2" t="s">
         <v>28</v>
       </c>
@@ -1218,22 +1270,22 @@
         <v>42</v>
       </c>
       <c r="I17" s="2"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="9"/>
       <c r="L17" s="2"/>
       <c r="P17" s="2"/>
-      <c r="Q17" s="7"/>
-      <c r="R17" s="8"/>
+      <c r="Q17" s="8"/>
+      <c r="R17" s="9"/>
       <c r="S17" s="2"/>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="8"/>
+      <c r="C18" s="9"/>
       <c r="D18" s="2" t="s">
         <v>23</v>
       </c>
@@ -1241,22 +1293,22 @@
         <v>42</v>
       </c>
       <c r="I18" s="2"/>
-      <c r="J18" s="7"/>
-      <c r="K18" s="8"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="9"/>
       <c r="L18" s="2"/>
       <c r="P18" s="2"/>
-      <c r="Q18" s="7"/>
-      <c r="R18" s="8"/>
+      <c r="Q18" s="8"/>
+      <c r="R18" s="9"/>
       <c r="S18" s="2"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="8"/>
+      <c r="C19" s="9"/>
       <c r="D19" s="2" t="s">
         <v>28</v>
       </c>
@@ -1264,22 +1316,22 @@
         <v>42</v>
       </c>
       <c r="I19" s="2"/>
-      <c r="J19" s="7"/>
-      <c r="K19" s="8"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="9"/>
       <c r="L19" s="2"/>
       <c r="P19" s="2"/>
-      <c r="Q19" s="7"/>
-      <c r="R19" s="8"/>
+      <c r="Q19" s="8"/>
+      <c r="R19" s="9"/>
       <c r="S19" s="2"/>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C20" s="8"/>
+      <c r="C20" s="9"/>
       <c r="D20" s="2" t="s">
         <v>35</v>
       </c>
@@ -1287,186 +1339,270 @@
         <v>42</v>
       </c>
       <c r="I20" s="2"/>
-      <c r="J20" s="7"/>
-      <c r="K20" s="8"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="9"/>
       <c r="L20" s="2"/>
       <c r="P20" s="2"/>
-      <c r="Q20" s="7"/>
-      <c r="R20" s="8"/>
+      <c r="Q20" s="8"/>
+      <c r="R20" s="9"/>
       <c r="S20" s="2"/>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="8"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="9"/>
       <c r="D21" s="2"/>
       <c r="I21" s="2"/>
-      <c r="J21" s="7"/>
-      <c r="K21" s="8"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="9"/>
       <c r="L21" s="2"/>
       <c r="P21" s="2"/>
-      <c r="Q21" s="7"/>
-      <c r="R21" s="8"/>
+      <c r="Q21" s="8"/>
+      <c r="R21" s="9"/>
       <c r="S21" s="2"/>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="8"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="9"/>
       <c r="D22" s="2"/>
       <c r="I22" s="2"/>
-      <c r="J22" s="7"/>
-      <c r="K22" s="8"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="9"/>
       <c r="L22" s="2"/>
       <c r="P22" s="2"/>
-      <c r="Q22" s="7"/>
-      <c r="R22" s="8"/>
+      <c r="Q22" s="8"/>
+      <c r="R22" s="9"/>
       <c r="S22" s="2"/>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="8"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="9"/>
       <c r="D23" s="2"/>
       <c r="I23" s="2"/>
-      <c r="J23" s="7"/>
-      <c r="K23" s="8"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="9"/>
       <c r="L23" s="2"/>
       <c r="P23" s="2"/>
-      <c r="Q23" s="7"/>
-      <c r="R23" s="8"/>
+      <c r="Q23" s="8"/>
+      <c r="R23" s="9"/>
       <c r="S23" s="2"/>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
-      <c r="B24" s="7"/>
-      <c r="C24" s="8"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="9"/>
       <c r="D24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="7"/>
-      <c r="K24" s="8"/>
+      <c r="J24" s="8"/>
+      <c r="K24" s="9"/>
       <c r="L24" s="2"/>
       <c r="P24" s="2"/>
-      <c r="Q24" s="7"/>
-      <c r="R24" s="8"/>
+      <c r="Q24" s="8"/>
+      <c r="R24" s="9"/>
       <c r="S24" s="2"/>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="7"/>
-      <c r="C25" s="8"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="9"/>
       <c r="D25" s="2"/>
       <c r="I25" s="2"/>
-      <c r="J25" s="7"/>
-      <c r="K25" s="8"/>
+      <c r="J25" s="8"/>
+      <c r="K25" s="9"/>
       <c r="L25" s="2"/>
       <c r="P25" s="2"/>
-      <c r="Q25" s="7"/>
-      <c r="R25" s="8"/>
+      <c r="Q25" s="8"/>
+      <c r="R25" s="9"/>
       <c r="S25" s="2"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
-      <c r="B26" s="7"/>
-      <c r="C26" s="8"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="9"/>
       <c r="D26" s="2"/>
       <c r="I26" s="2"/>
-      <c r="J26" s="7"/>
-      <c r="K26" s="8"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="9"/>
       <c r="L26" s="2"/>
       <c r="P26" s="2"/>
-      <c r="Q26" s="7"/>
-      <c r="R26" s="8"/>
+      <c r="Q26" s="8"/>
+      <c r="R26" s="9"/>
       <c r="S26" s="2"/>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="7"/>
-      <c r="C27" s="8"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="9"/>
       <c r="D27" s="2"/>
       <c r="I27" s="2"/>
-      <c r="J27" s="7"/>
-      <c r="K27" s="8"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="9"/>
       <c r="L27" s="2"/>
       <c r="P27" s="2"/>
-      <c r="Q27" s="7"/>
-      <c r="R27" s="8"/>
+      <c r="Q27" s="8"/>
+      <c r="R27" s="9"/>
       <c r="S27" s="2"/>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
-      <c r="B28" s="7"/>
-      <c r="C28" s="8"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="9"/>
       <c r="D28" s="2"/>
       <c r="I28" s="2"/>
-      <c r="J28" s="7"/>
-      <c r="K28" s="8"/>
+      <c r="J28" s="8"/>
+      <c r="K28" s="9"/>
       <c r="L28" s="2"/>
       <c r="P28" s="2"/>
-      <c r="Q28" s="7"/>
-      <c r="R28" s="8"/>
+      <c r="Q28" s="8"/>
+      <c r="R28" s="9"/>
       <c r="S28" s="2"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
-      <c r="B29" s="7"/>
-      <c r="C29" s="8"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="9"/>
       <c r="D29" s="2"/>
       <c r="I29" s="2"/>
-      <c r="J29" s="7"/>
-      <c r="K29" s="8"/>
+      <c r="J29" s="8"/>
+      <c r="K29" s="9"/>
       <c r="L29" s="2"/>
       <c r="P29" s="2"/>
-      <c r="Q29" s="7"/>
-      <c r="R29" s="8"/>
+      <c r="Q29" s="8"/>
+      <c r="R29" s="9"/>
       <c r="S29" s="2"/>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
-      <c r="B30" s="7"/>
-      <c r="C30" s="8"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="9"/>
       <c r="D30" s="2"/>
       <c r="I30" s="2"/>
-      <c r="J30" s="7"/>
-      <c r="K30" s="8"/>
+      <c r="J30" s="8"/>
+      <c r="K30" s="9"/>
       <c r="L30" s="2"/>
       <c r="P30" s="2"/>
-      <c r="Q30" s="7"/>
-      <c r="R30" s="8"/>
+      <c r="Q30" s="8"/>
+      <c r="R30" s="9"/>
       <c r="S30" s="2"/>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
-      <c r="B31" s="9"/>
-      <c r="C31" s="10"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="11"/>
       <c r="D31" s="3"/>
       <c r="I31" s="3"/>
-      <c r="J31" s="9"/>
-      <c r="K31" s="10"/>
+      <c r="J31" s="10"/>
+      <c r="K31" s="11"/>
       <c r="L31" s="3"/>
       <c r="P31" s="3"/>
-      <c r="Q31" s="9"/>
-      <c r="R31" s="10"/>
+      <c r="Q31" s="10"/>
+      <c r="R31" s="11"/>
       <c r="S31" s="3"/>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="22"/>
-      <c r="C32" s="22"/>
+      <c r="B32" s="7"/>
+      <c r="C32" s="7"/>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B33" s="22"/>
-      <c r="C33" s="22"/>
+      <c r="B33" s="7"/>
+      <c r="C33" s="7"/>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B34" s="22"/>
-      <c r="C34" s="22"/>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7"/>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B35" s="22"/>
-      <c r="C35" s="22"/>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="100">
+    <mergeCell ref="Q30:R30"/>
+    <mergeCell ref="Q31:R31"/>
+    <mergeCell ref="Q25:R25"/>
+    <mergeCell ref="Q26:R26"/>
+    <mergeCell ref="Q27:R27"/>
+    <mergeCell ref="Q28:R28"/>
+    <mergeCell ref="Q29:R29"/>
+    <mergeCell ref="Q20:R20"/>
+    <mergeCell ref="Q21:R21"/>
+    <mergeCell ref="Q22:R22"/>
+    <mergeCell ref="Q23:R23"/>
+    <mergeCell ref="Q24:R24"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="Q16:R16"/>
+    <mergeCell ref="Q17:R17"/>
+    <mergeCell ref="Q18:R18"/>
+    <mergeCell ref="Q19:R19"/>
+    <mergeCell ref="Q10:R10"/>
+    <mergeCell ref="Q11:R11"/>
+    <mergeCell ref="Q12:R12"/>
+    <mergeCell ref="Q13:R13"/>
+    <mergeCell ref="Q14:R14"/>
+    <mergeCell ref="Q5:R5"/>
+    <mergeCell ref="Q6:R6"/>
+    <mergeCell ref="Q7:R7"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="Q9:R9"/>
+    <mergeCell ref="P1:S1"/>
+    <mergeCell ref="P2:S2"/>
+    <mergeCell ref="P3:Q3"/>
+    <mergeCell ref="R3:S3"/>
+    <mergeCell ref="Q4:S4"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="I1:L1"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B31:C31"/>
@@ -1483,90 +1619,6 @@
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="I1:L1"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="P1:S1"/>
-    <mergeCell ref="P2:S2"/>
-    <mergeCell ref="P3:Q3"/>
-    <mergeCell ref="R3:S3"/>
-    <mergeCell ref="Q4:S4"/>
-    <mergeCell ref="Q5:R5"/>
-    <mergeCell ref="Q6:R6"/>
-    <mergeCell ref="Q7:R7"/>
-    <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="Q9:R9"/>
-    <mergeCell ref="Q10:R10"/>
-    <mergeCell ref="Q11:R11"/>
-    <mergeCell ref="Q12:R12"/>
-    <mergeCell ref="Q13:R13"/>
-    <mergeCell ref="Q14:R14"/>
-    <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="Q16:R16"/>
-    <mergeCell ref="Q17:R17"/>
-    <mergeCell ref="Q18:R18"/>
-    <mergeCell ref="Q19:R19"/>
-    <mergeCell ref="Q20:R20"/>
-    <mergeCell ref="Q21:R21"/>
-    <mergeCell ref="Q22:R22"/>
-    <mergeCell ref="Q23:R23"/>
-    <mergeCell ref="Q24:R24"/>
-    <mergeCell ref="Q30:R30"/>
-    <mergeCell ref="Q31:R31"/>
-    <mergeCell ref="Q25:R25"/>
-    <mergeCell ref="Q26:R26"/>
-    <mergeCell ref="Q27:R27"/>
-    <mergeCell ref="Q28:R28"/>
-    <mergeCell ref="Q29:R29"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat:integrate docx report generation and refine analysis workflow - **Report Generator**: Refactored  to generate  files using a new , moving away from markdown-based templates. - **Workflow & Prompts**: Added new system prompts for  and . Updated the AWS Step Functions state machine () and SAM  to align with the new analysis process. - **S3 & Storage**: Cleaned up  and added job progress functionality in . - **Frontend**: Updated  and  to handle the new document generation states and outputs. - **Testing**: Introduced comprehensive smoke tests () and template filler tests () with new  and  fixtures. - **Clean up**: Removed obsolete markdown templates (, , ) and updated CI/CD workflows.
</commit_message>
<xml_diff>
--- a/llms_calls_accounting.xlsx
+++ b/llms_calls_accounting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\03_iastronauts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8CC3B22-24CB-45DF-8265-1C0E63A78934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{771B9224-F0D3-4325-8913-3B5B0C54C738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{59B62FDA-1497-4401-82EC-1B2F7D702BCC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="59">
   <si>
     <t>Consumo Tokens CreditIQ</t>
   </si>
@@ -186,6 +186,36 @@
   </si>
   <si>
     <t>2026-05-31:13:35</t>
+  </si>
+  <si>
+    <t>0.02</t>
+  </si>
+  <si>
+    <t>P.INMOBILIARIO</t>
+  </si>
+  <si>
+    <t>2026-05-30:18:32</t>
+  </si>
+  <si>
+    <t>0.2</t>
+  </si>
+  <si>
+    <t>2026-05-30:18:39</t>
+  </si>
+  <si>
+    <t>2026-05-30:18:48</t>
+  </si>
+  <si>
+    <t>Document Generator + Review</t>
+  </si>
+  <si>
+    <t>2026-05-30:18:52</t>
+  </si>
+  <si>
+    <t>2026-05-30:20:11</t>
+  </si>
+  <si>
+    <t>Document Generator</t>
   </si>
 </sst>
 </file>
@@ -390,6 +420,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -405,6 +436,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -437,13 +474,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -789,130 +819,131 @@
     <col min="9" max="9" width="15.42578125" customWidth="1"/>
     <col min="11" max="11" width="15.85546875" customWidth="1"/>
     <col min="12" max="12" width="17.85546875" customWidth="1"/>
-    <col min="16" max="16" width="17.140625" customWidth="1"/>
-    <col min="18" max="18" width="16.85546875" customWidth="1"/>
+    <col min="16" max="16" width="19.42578125" customWidth="1"/>
+    <col min="18" max="18" width="18.28515625" customWidth="1"/>
+    <col min="19" max="19" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="I1" s="22" t="s">
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="I1" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="P1" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
-      <c r="S1" s="22"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="P1" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q1" s="25"/>
+      <c r="R1" s="25"/>
+      <c r="S1" s="25"/>
     </row>
     <row r="2" spans="1:20" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="14"/>
-      <c r="I2" s="12" t="s">
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="17"/>
+      <c r="I2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="J2" s="13"/>
-      <c r="K2" s="13"/>
-      <c r="L2" s="14"/>
-      <c r="P2" s="12" t="s">
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="17"/>
+      <c r="P2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="Q2" s="13"/>
-      <c r="R2" s="13"/>
-      <c r="S2" s="14"/>
+      <c r="Q2" s="16"/>
+      <c r="R2" s="16"/>
+      <c r="S2" s="17"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="15" t="s">
+      <c r="B3" s="19"/>
+      <c r="C3" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="16"/>
-      <c r="I3" s="15" t="s">
+      <c r="D3" s="19"/>
+      <c r="I3" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="16"/>
-      <c r="K3" s="15" t="s">
+      <c r="J3" s="19"/>
+      <c r="K3" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="16"/>
-      <c r="P3" s="15" t="s">
+      <c r="L3" s="19"/>
+      <c r="P3" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="Q3" s="16"/>
-      <c r="R3" s="15" t="s">
+      <c r="Q3" s="19"/>
+      <c r="R3" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="S3" s="16"/>
+      <c r="S3" s="19"/>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="20"/>
-      <c r="D4" s="21"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="24"/>
       <c r="I4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="19" t="s">
+      <c r="J4" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="20"/>
-      <c r="L4" s="21"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="24"/>
       <c r="P4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="Q4" s="19" t="s">
+      <c r="Q4" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="R4" s="20"/>
-      <c r="S4" s="21"/>
+      <c r="R4" s="23"/>
+      <c r="S4" s="24"/>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="18"/>
+      <c r="C5" s="21"/>
       <c r="D5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="17" t="s">
+      <c r="J5" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="K5" s="18"/>
+      <c r="K5" s="21"/>
       <c r="L5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="P5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="Q5" s="17" t="s">
+      <c r="Q5" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="R5" s="18"/>
+      <c r="R5" s="21"/>
       <c r="S5" s="4" t="s">
         <v>8</v>
       </c>
@@ -921,10 +952,10 @@
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="9"/>
+      <c r="C6" s="10"/>
       <c r="D6" s="2" t="s">
         <v>10</v>
       </c>
@@ -934,10 +965,10 @@
       <c r="I6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="K6" s="9"/>
+      <c r="K6" s="10"/>
       <c r="L6" s="2" t="s">
         <v>35</v>
       </c>
@@ -947,10 +978,10 @@
       <c r="P6" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="Q6" s="8" t="s">
+      <c r="Q6" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="R6" s="9"/>
+      <c r="R6" s="10"/>
       <c r="S6" s="2" t="s">
         <v>23</v>
       </c>
@@ -962,10 +993,10 @@
       <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="9"/>
+      <c r="C7" s="10"/>
       <c r="D7" s="2" t="s">
         <v>11</v>
       </c>
@@ -975,10 +1006,10 @@
       <c r="I7" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="J7" s="8" t="s">
+      <c r="J7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="K7" s="9"/>
+      <c r="K7" s="10"/>
       <c r="L7" s="2" t="s">
         <v>37</v>
       </c>
@@ -988,10 +1019,10 @@
       <c r="P7" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="Q7" s="8" t="s">
+      <c r="Q7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="R7" s="9"/>
+      <c r="R7" s="10"/>
       <c r="S7" s="2" t="s">
         <v>44</v>
       </c>
@@ -1003,10 +1034,10 @@
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="9"/>
+      <c r="C8" s="10"/>
       <c r="D8" s="2" t="s">
         <v>10</v>
       </c>
@@ -1016,10 +1047,10 @@
       <c r="I8" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="K8" s="9"/>
+      <c r="K8" s="10"/>
       <c r="L8" s="2" t="s">
         <v>23</v>
       </c>
@@ -1029,12 +1060,12 @@
       <c r="P8" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="Q8" s="8" t="s">
+      <c r="Q8" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="R8" s="9"/>
+      <c r="R8" s="10"/>
       <c r="S8" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="T8" t="s">
         <v>42</v>
@@ -1044,10 +1075,10 @@
       <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="9"/>
+      <c r="C9" s="10"/>
       <c r="D9" s="2" t="s">
         <v>16</v>
       </c>
@@ -1057,29 +1088,38 @@
       <c r="I9" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="J9" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="K9" s="9"/>
+      <c r="K9" s="10"/>
       <c r="L9" s="2" t="s">
         <v>28</v>
       </c>
       <c r="M9" t="s">
         <v>42</v>
       </c>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="8"/>
-      <c r="R9" s="9"/>
-      <c r="S9" s="2"/>
+      <c r="P9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="R9" s="10"/>
+      <c r="S9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="T9" s="6" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="9"/>
+      <c r="C10" s="10"/>
       <c r="D10" s="2" t="s">
         <v>10</v>
       </c>
@@ -1089,29 +1129,38 @@
       <c r="I10" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="J10" s="8" t="s">
+      <c r="J10" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="K10" s="9"/>
+      <c r="K10" s="10"/>
       <c r="L10" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M10" t="s">
         <v>42</v>
       </c>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="8"/>
-      <c r="R10" s="9"/>
-      <c r="S10" s="2"/>
+      <c r="P10" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q10" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="R10" s="10"/>
+      <c r="S10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="T10" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="9"/>
+      <c r="C11" s="10"/>
       <c r="D11" s="2" t="s">
         <v>18</v>
       </c>
@@ -1121,29 +1170,38 @@
       <c r="I11" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="J11" s="8" t="s">
+      <c r="J11" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="K11" s="9"/>
+      <c r="K11" s="10"/>
       <c r="L11" s="2" t="s">
         <v>46</v>
       </c>
       <c r="M11" t="s">
         <v>42</v>
       </c>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="8"/>
-      <c r="R11" s="9"/>
-      <c r="S11" s="2"/>
+      <c r="P11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q11" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="R11" s="10"/>
+      <c r="S11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="T11" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="9"/>
+      <c r="C12" s="10"/>
       <c r="D12" s="2" t="s">
         <v>10</v>
       </c>
@@ -1151,22 +1209,31 @@
         <v>42</v>
       </c>
       <c r="I12" s="2"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="10"/>
       <c r="L12" s="2"/>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="8"/>
-      <c r="R12" s="9"/>
-      <c r="S12" s="2"/>
+      <c r="P12" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q12" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="R12" s="10"/>
+      <c r="S12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="T12" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="9"/>
+      <c r="C13" s="10"/>
       <c r="D13" s="2" t="s">
         <v>22</v>
       </c>
@@ -1174,23 +1241,32 @@
         <v>42</v>
       </c>
       <c r="I13" s="2"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="10"/>
       <c r="L13" s="2"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="8"/>
-      <c r="R13" s="9"/>
-      <c r="S13" s="2"/>
+      <c r="P13" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q13" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="R13" s="10"/>
+      <c r="S13" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="T13" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="25"/>
-      <c r="D14" s="23" t="s">
+      <c r="C14" s="14"/>
+      <c r="D14" s="7" t="s">
         <v>23</v>
       </c>
       <c r="E14" s="5" t="s">
@@ -1201,22 +1277,31 @@
       </c>
       <c r="G14" s="5"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="8"/>
-      <c r="K14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="10"/>
       <c r="L14" s="2"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="8"/>
-      <c r="R14" s="9"/>
-      <c r="S14" s="2"/>
+      <c r="P14" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q14" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="R14" s="10"/>
+      <c r="S14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="T14" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="9"/>
+      <c r="C15" s="10"/>
       <c r="D15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1224,22 +1309,22 @@
         <v>42</v>
       </c>
       <c r="I15" s="2"/>
-      <c r="J15" s="8"/>
-      <c r="K15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="10"/>
       <c r="L15" s="2"/>
       <c r="P15" s="2"/>
-      <c r="Q15" s="8"/>
-      <c r="R15" s="9"/>
+      <c r="Q15" s="9"/>
+      <c r="R15" s="10"/>
       <c r="S15" s="2"/>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="9"/>
+      <c r="C16" s="10"/>
       <c r="D16" s="2" t="s">
         <v>23</v>
       </c>
@@ -1247,22 +1332,22 @@
         <v>42</v>
       </c>
       <c r="I16" s="2"/>
-      <c r="J16" s="8"/>
-      <c r="K16" s="9"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="10"/>
       <c r="L16" s="2"/>
       <c r="P16" s="2"/>
-      <c r="Q16" s="8"/>
-      <c r="R16" s="9"/>
+      <c r="Q16" s="9"/>
+      <c r="R16" s="10"/>
       <c r="S16" s="2"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C17" s="9"/>
+      <c r="C17" s="10"/>
       <c r="D17" s="2" t="s">
         <v>28</v>
       </c>
@@ -1270,22 +1355,22 @@
         <v>42</v>
       </c>
       <c r="I17" s="2"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="9"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="10"/>
       <c r="L17" s="2"/>
       <c r="P17" s="2"/>
-      <c r="Q17" s="8"/>
-      <c r="R17" s="9"/>
+      <c r="Q17" s="9"/>
+      <c r="R17" s="10"/>
       <c r="S17" s="2"/>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="9"/>
+      <c r="C18" s="10"/>
       <c r="D18" s="2" t="s">
         <v>23</v>
       </c>
@@ -1293,22 +1378,22 @@
         <v>42</v>
       </c>
       <c r="I18" s="2"/>
-      <c r="J18" s="8"/>
-      <c r="K18" s="9"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="10"/>
       <c r="L18" s="2"/>
       <c r="P18" s="2"/>
-      <c r="Q18" s="8"/>
-      <c r="R18" s="9"/>
+      <c r="Q18" s="9"/>
+      <c r="R18" s="10"/>
       <c r="S18" s="2"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="9"/>
+      <c r="C19" s="10"/>
       <c r="D19" s="2" t="s">
         <v>28</v>
       </c>
@@ -1316,22 +1401,22 @@
         <v>42</v>
       </c>
       <c r="I19" s="2"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="9"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="10"/>
       <c r="L19" s="2"/>
       <c r="P19" s="2"/>
-      <c r="Q19" s="8"/>
-      <c r="R19" s="9"/>
+      <c r="Q19" s="9"/>
+      <c r="R19" s="10"/>
       <c r="S19" s="2"/>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C20" s="9"/>
+      <c r="C20" s="10"/>
       <c r="D20" s="2" t="s">
         <v>35</v>
       </c>
@@ -1339,183 +1424,183 @@
         <v>42</v>
       </c>
       <c r="I20" s="2"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="9"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="10"/>
       <c r="L20" s="2"/>
       <c r="P20" s="2"/>
-      <c r="Q20" s="8"/>
-      <c r="R20" s="9"/>
+      <c r="Q20" s="9"/>
+      <c r="R20" s="10"/>
       <c r="S20" s="2"/>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="9"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="10"/>
       <c r="D21" s="2"/>
       <c r="I21" s="2"/>
-      <c r="J21" s="8"/>
-      <c r="K21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="10"/>
       <c r="L21" s="2"/>
       <c r="P21" s="2"/>
-      <c r="Q21" s="8"/>
-      <c r="R21" s="9"/>
+      <c r="Q21" s="9"/>
+      <c r="R21" s="10"/>
       <c r="S21" s="2"/>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="9"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="10"/>
       <c r="D22" s="2"/>
       <c r="I22" s="2"/>
-      <c r="J22" s="8"/>
-      <c r="K22" s="9"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="10"/>
       <c r="L22" s="2"/>
       <c r="P22" s="2"/>
-      <c r="Q22" s="8"/>
-      <c r="R22" s="9"/>
+      <c r="Q22" s="9"/>
+      <c r="R22" s="10"/>
       <c r="S22" s="2"/>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="9"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="10"/>
       <c r="D23" s="2"/>
       <c r="I23" s="2"/>
-      <c r="J23" s="8"/>
-      <c r="K23" s="9"/>
+      <c r="J23" s="9"/>
+      <c r="K23" s="10"/>
       <c r="L23" s="2"/>
       <c r="P23" s="2"/>
-      <c r="Q23" s="8"/>
-      <c r="R23" s="9"/>
+      <c r="Q23" s="9"/>
+      <c r="R23" s="10"/>
       <c r="S23" s="2"/>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
-      <c r="B24" s="8"/>
-      <c r="C24" s="9"/>
+      <c r="B24" s="9"/>
+      <c r="C24" s="10"/>
       <c r="D24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="8"/>
-      <c r="K24" s="9"/>
+      <c r="J24" s="9"/>
+      <c r="K24" s="10"/>
       <c r="L24" s="2"/>
       <c r="P24" s="2"/>
-      <c r="Q24" s="8"/>
-      <c r="R24" s="9"/>
+      <c r="Q24" s="9"/>
+      <c r="R24" s="10"/>
       <c r="S24" s="2"/>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="9"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="10"/>
       <c r="D25" s="2"/>
       <c r="I25" s="2"/>
-      <c r="J25" s="8"/>
-      <c r="K25" s="9"/>
+      <c r="J25" s="9"/>
+      <c r="K25" s="10"/>
       <c r="L25" s="2"/>
       <c r="P25" s="2"/>
-      <c r="Q25" s="8"/>
-      <c r="R25" s="9"/>
+      <c r="Q25" s="9"/>
+      <c r="R25" s="10"/>
       <c r="S25" s="2"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="9"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="10"/>
       <c r="D26" s="2"/>
       <c r="I26" s="2"/>
-      <c r="J26" s="8"/>
-      <c r="K26" s="9"/>
+      <c r="J26" s="9"/>
+      <c r="K26" s="10"/>
       <c r="L26" s="2"/>
       <c r="P26" s="2"/>
-      <c r="Q26" s="8"/>
-      <c r="R26" s="9"/>
+      <c r="Q26" s="9"/>
+      <c r="R26" s="10"/>
       <c r="S26" s="2"/>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="8"/>
-      <c r="C27" s="9"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="10"/>
       <c r="D27" s="2"/>
       <c r="I27" s="2"/>
-      <c r="J27" s="8"/>
-      <c r="K27" s="9"/>
+      <c r="J27" s="9"/>
+      <c r="K27" s="10"/>
       <c r="L27" s="2"/>
       <c r="P27" s="2"/>
-      <c r="Q27" s="8"/>
-      <c r="R27" s="9"/>
+      <c r="Q27" s="9"/>
+      <c r="R27" s="10"/>
       <c r="S27" s="2"/>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="9"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="10"/>
       <c r="D28" s="2"/>
       <c r="I28" s="2"/>
-      <c r="J28" s="8"/>
-      <c r="K28" s="9"/>
+      <c r="J28" s="9"/>
+      <c r="K28" s="10"/>
       <c r="L28" s="2"/>
       <c r="P28" s="2"/>
-      <c r="Q28" s="8"/>
-      <c r="R28" s="9"/>
+      <c r="Q28" s="9"/>
+      <c r="R28" s="10"/>
       <c r="S28" s="2"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="9"/>
+      <c r="B29" s="9"/>
+      <c r="C29" s="10"/>
       <c r="D29" s="2"/>
       <c r="I29" s="2"/>
-      <c r="J29" s="8"/>
-      <c r="K29" s="9"/>
+      <c r="J29" s="9"/>
+      <c r="K29" s="10"/>
       <c r="L29" s="2"/>
       <c r="P29" s="2"/>
-      <c r="Q29" s="8"/>
-      <c r="R29" s="9"/>
+      <c r="Q29" s="9"/>
+      <c r="R29" s="10"/>
       <c r="S29" s="2"/>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
-      <c r="B30" s="8"/>
-      <c r="C30" s="9"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="10"/>
       <c r="D30" s="2"/>
       <c r="I30" s="2"/>
-      <c r="J30" s="8"/>
-      <c r="K30" s="9"/>
+      <c r="J30" s="9"/>
+      <c r="K30" s="10"/>
       <c r="L30" s="2"/>
       <c r="P30" s="2"/>
-      <c r="Q30" s="8"/>
-      <c r="R30" s="9"/>
+      <c r="Q30" s="9"/>
+      <c r="R30" s="10"/>
       <c r="S30" s="2"/>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="11"/>
+      <c r="B31" s="11"/>
+      <c r="C31" s="12"/>
       <c r="D31" s="3"/>
       <c r="I31" s="3"/>
-      <c r="J31" s="10"/>
-      <c r="K31" s="11"/>
+      <c r="J31" s="11"/>
+      <c r="K31" s="12"/>
       <c r="L31" s="3"/>
       <c r="P31" s="3"/>
-      <c r="Q31" s="10"/>
-      <c r="R31" s="11"/>
+      <c r="Q31" s="11"/>
+      <c r="R31" s="12"/>
       <c r="S31" s="3"/>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="7"/>
-      <c r="C32" s="7"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B33" s="7"/>
-      <c r="C33" s="7"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="8"/>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B34" s="7"/>
-      <c r="C34" s="7"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="8"/>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B35" s="7"/>
-      <c r="C35" s="7"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="100">
@@ -1622,5 +1707,6 @@
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Implement fund policy engine, management reporting, and NIIF validations
This commit introduces several major enhancements to the extraction and analysis pipelines, including comprehensive support for fund policies, management reports, and cost-optimized LLM routing.

Key changes include:
- Agents & Analyzers:
  - Added  and  for fund policy evaluations.
  - Added new  agent and associated prompt ().
  - Implemented NIIF validation logic ( and ).
  - Improved , , and introduced  for advanced risk scoring.
  - Enhanced , , and  handlers.
- Shared Logic & Models:
  - Expanded  and added .
  - Significant updates to  to support LLM cost tracking and optimization, alongside new test coverage.
  - Extended core data models for analyzers, extractors, reports, and scorers.
- Frontend:
  - Major UI updates to  to surface new analysis results, scores, and management reports.
- Configuration & Infrastructure:
  - Updated SAM  and .
  - Updated  with current project guidelines and tasks.
</commit_message>
<xml_diff>
--- a/llms_calls_accounting.xlsx
+++ b/llms_calls_accounting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\03_iastronauts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F024FFC-9414-442B-A63F-8318F1EA905B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59EEA947-1DEC-4F3D-9856-0523DA9FE88A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{59B62FDA-1497-4401-82EC-1B2F7D702BCC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="104">
   <si>
     <t>Consumo Tokens CreditIQ</t>
   </si>
@@ -345,6 +345,12 @@
   </si>
   <si>
     <t>2026-06-02:22:17</t>
+  </si>
+  <si>
+    <t>2026-06-05:15:58</t>
+  </si>
+  <si>
+    <t>2026-06-05:22:16</t>
   </si>
 </sst>
 </file>
@@ -571,10 +577,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -586,11 +598,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -601,19 +613,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -950,7 +956,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B052F0D6-0E50-4E03-8DA0-D70F625DE32B}">
-  <dimension ref="A1:T59"/>
+  <dimension ref="A1:T64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.85546875" customWidth="1"/>
@@ -966,125 +972,125 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="I1" s="29" t="s">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="I1" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="P1" s="29" t="s">
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="P1" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="Q1" s="29"/>
-      <c r="R1" s="29"/>
-      <c r="S1" s="29"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
     </row>
     <row r="2" spans="1:20" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="24"/>
-      <c r="I2" s="22" t="s">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="26"/>
+      <c r="I2" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="24"/>
-      <c r="P2" s="22" t="s">
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="26"/>
+      <c r="P2" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="24"/>
+      <c r="Q2" s="25"/>
+      <c r="R2" s="25"/>
+      <c r="S2" s="26"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="25" t="s">
+      <c r="B3" s="18"/>
+      <c r="C3" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="26"/>
-      <c r="I3" s="25" t="s">
+      <c r="D3" s="18"/>
+      <c r="I3" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="26"/>
-      <c r="K3" s="25" t="s">
+      <c r="J3" s="18"/>
+      <c r="K3" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="26"/>
-      <c r="P3" s="25" t="s">
+      <c r="L3" s="18"/>
+      <c r="P3" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="Q3" s="26"/>
-      <c r="R3" s="25" t="s">
+      <c r="Q3" s="18"/>
+      <c r="R3" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="S3" s="26"/>
+      <c r="S3" s="18"/>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="18"/>
-      <c r="D4" s="19"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="21"/>
       <c r="I4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="17" t="s">
+      <c r="J4" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="18"/>
-      <c r="L4" s="19"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="21"/>
       <c r="P4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="Q4" s="17" t="s">
+      <c r="Q4" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="R4" s="18"/>
-      <c r="S4" s="19"/>
+      <c r="R4" s="20"/>
+      <c r="S4" s="21"/>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="28"/>
+      <c r="C5" s="23"/>
       <c r="D5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="27" t="s">
+      <c r="J5" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="K5" s="28"/>
+      <c r="K5" s="23"/>
       <c r="L5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="P5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="Q5" s="27" t="s">
+      <c r="Q5" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="R5" s="28"/>
+      <c r="R5" s="23"/>
       <c r="S5" s="4" t="s">
         <v>8</v>
       </c>
@@ -1421,10 +1427,10 @@
       <c r="A14" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="21"/>
+      <c r="C14" s="16"/>
       <c r="D14" s="7" t="s">
         <v>23</v>
       </c>
@@ -2303,10 +2309,19 @@
       <c r="S47" s="2"/>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A48" s="2"/>
-      <c r="B48" s="15"/>
-      <c r="C48" s="16"/>
-      <c r="D48" s="2"/>
+      <c r="A48" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B48" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C48" s="12"/>
+      <c r="D48" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E48" t="s">
+        <v>42</v>
+      </c>
       <c r="I48" s="2"/>
       <c r="J48" s="8"/>
       <c r="K48" s="9"/>
@@ -2317,10 +2332,19 @@
       <c r="S48" s="2"/>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A49" s="2"/>
-      <c r="B49" s="15"/>
-      <c r="C49" s="16"/>
-      <c r="D49" s="2"/>
+      <c r="A49" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B49" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C49" s="12"/>
+      <c r="D49" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E49" t="s">
+        <v>42</v>
+      </c>
       <c r="I49" s="2"/>
       <c r="J49" s="8"/>
       <c r="K49" s="9"/>
@@ -2332,8 +2356,8 @@
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A50" s="2"/>
-      <c r="B50" s="15"/>
-      <c r="C50" s="16"/>
+      <c r="B50" s="28"/>
+      <c r="C50" s="29"/>
       <c r="D50" s="2"/>
       <c r="I50" s="2"/>
       <c r="J50" s="8"/>
@@ -2346,8 +2370,8 @@
     </row>
     <row r="51" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A51" s="2"/>
-      <c r="B51" s="15"/>
-      <c r="C51" s="16"/>
+      <c r="B51" s="28"/>
+      <c r="C51" s="29"/>
       <c r="D51" s="2"/>
       <c r="I51" s="2"/>
       <c r="J51" s="8"/>
@@ -2360,8 +2384,8 @@
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="2"/>
-      <c r="B52" s="15"/>
-      <c r="C52" s="16"/>
+      <c r="B52" s="28"/>
+      <c r="C52" s="29"/>
       <c r="D52" s="2"/>
       <c r="I52" s="2"/>
       <c r="J52" s="8"/>
@@ -2374,70 +2398,140 @@
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A53" s="2"/>
-      <c r="B53" s="15"/>
-      <c r="C53" s="16"/>
+      <c r="B53" s="28"/>
+      <c r="C53" s="29"/>
       <c r="D53" s="2"/>
       <c r="I53" s="2"/>
-      <c r="J53" s="11"/>
-      <c r="K53" s="12"/>
+      <c r="J53" s="8"/>
+      <c r="K53" s="9"/>
       <c r="L53" s="2"/>
       <c r="P53" s="2"/>
-      <c r="Q53" s="11"/>
-      <c r="R53" s="12"/>
+      <c r="Q53" s="8"/>
+      <c r="R53" s="9"/>
       <c r="S53" s="2"/>
     </row>
     <row r="54" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="2"/>
-      <c r="B54" s="11"/>
-      <c r="C54" s="12"/>
+      <c r="B54" s="28"/>
+      <c r="C54" s="29"/>
       <c r="D54" s="2"/>
       <c r="I54" s="2"/>
-      <c r="J54" s="11"/>
-      <c r="K54" s="12"/>
+      <c r="J54" s="8"/>
+      <c r="K54" s="9"/>
       <c r="L54" s="2"/>
       <c r="P54" s="2"/>
-      <c r="Q54" s="11"/>
-      <c r="R54" s="12"/>
+      <c r="Q54" s="8"/>
+      <c r="R54" s="9"/>
       <c r="S54" s="2"/>
     </row>
     <row r="55" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A55" s="3"/>
-      <c r="B55" s="13"/>
-      <c r="C55" s="14"/>
-      <c r="D55" s="3"/>
-      <c r="I55" s="3"/>
-      <c r="J55" s="13"/>
-      <c r="K55" s="14"/>
-      <c r="L55" s="3"/>
-      <c r="P55" s="3"/>
-      <c r="Q55" s="13"/>
-      <c r="R55" s="14"/>
-      <c r="S55" s="3"/>
+      <c r="A55" s="2"/>
+      <c r="B55" s="28"/>
+      <c r="C55" s="29"/>
+      <c r="D55" s="2"/>
+      <c r="I55" s="2"/>
+      <c r="J55" s="8"/>
+      <c r="K55" s="9"/>
+      <c r="L55" s="2"/>
+      <c r="P55" s="2"/>
+      <c r="Q55" s="8"/>
+      <c r="R55" s="9"/>
+      <c r="S55" s="2"/>
     </row>
     <row r="56" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B56" s="10"/>
-      <c r="C56" s="10"/>
+      <c r="A56" s="2"/>
+      <c r="B56" s="28"/>
+      <c r="C56" s="29"/>
+      <c r="D56" s="2"/>
+      <c r="I56" s="2"/>
+      <c r="J56" s="8"/>
+      <c r="K56" s="9"/>
+      <c r="L56" s="2"/>
+      <c r="P56" s="2"/>
+      <c r="Q56" s="8"/>
+      <c r="R56" s="9"/>
+      <c r="S56" s="2"/>
     </row>
     <row r="57" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B57" s="10"/>
-      <c r="C57" s="10"/>
+      <c r="A57" s="2"/>
+      <c r="B57" s="28"/>
+      <c r="C57" s="29"/>
+      <c r="D57" s="2"/>
+      <c r="I57" s="2"/>
+      <c r="J57" s="8"/>
+      <c r="K57" s="9"/>
+      <c r="L57" s="2"/>
+      <c r="P57" s="2"/>
+      <c r="Q57" s="8"/>
+      <c r="R57" s="9"/>
+      <c r="S57" s="2"/>
     </row>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B58" s="10"/>
-      <c r="C58" s="10"/>
+      <c r="A58" s="2"/>
+      <c r="B58" s="28"/>
+      <c r="C58" s="29"/>
+      <c r="D58" s="2"/>
+      <c r="I58" s="2"/>
+      <c r="J58" s="11"/>
+      <c r="K58" s="12"/>
+      <c r="L58" s="2"/>
+      <c r="P58" s="2"/>
+      <c r="Q58" s="11"/>
+      <c r="R58" s="12"/>
+      <c r="S58" s="2"/>
     </row>
     <row r="59" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B59" s="10"/>
-      <c r="C59" s="10"/>
+      <c r="A59" s="2"/>
+      <c r="B59" s="11"/>
+      <c r="C59" s="12"/>
+      <c r="D59" s="2"/>
+      <c r="I59" s="2"/>
+      <c r="J59" s="11"/>
+      <c r="K59" s="12"/>
+      <c r="L59" s="2"/>
+      <c r="P59" s="2"/>
+      <c r="Q59" s="11"/>
+      <c r="R59" s="12"/>
+      <c r="S59" s="2"/>
+    </row>
+    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A60" s="3"/>
+      <c r="B60" s="13"/>
+      <c r="C60" s="14"/>
+      <c r="D60" s="3"/>
+      <c r="I60" s="3"/>
+      <c r="J60" s="13"/>
+      <c r="K60" s="14"/>
+      <c r="L60" s="3"/>
+      <c r="P60" s="3"/>
+      <c r="Q60" s="13"/>
+      <c r="R60" s="14"/>
+      <c r="S60" s="3"/>
+    </row>
+    <row r="61" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B61" s="10"/>
+      <c r="C61" s="10"/>
+    </row>
+    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B62" s="10"/>
+      <c r="C62" s="10"/>
+    </row>
+    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B63" s="10"/>
+      <c r="C63" s="10"/>
+    </row>
+    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B64" s="10"/>
+      <c r="C64" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="138">
+  <mergeCells count="143">
     <mergeCell ref="J32:K32"/>
     <mergeCell ref="J33:K33"/>
     <mergeCell ref="J34:K34"/>
     <mergeCell ref="J35:K35"/>
     <mergeCell ref="J36:K36"/>
-    <mergeCell ref="J53:K53"/>
+    <mergeCell ref="J58:K58"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="B32:C32"/>
@@ -2447,12 +2541,17 @@
     <mergeCell ref="B46:C46"/>
     <mergeCell ref="B47:C47"/>
     <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="B57:C57"/>
     <mergeCell ref="B49:C49"/>
     <mergeCell ref="B50:C50"/>
     <mergeCell ref="B51:C51"/>
     <mergeCell ref="B52:C52"/>
-    <mergeCell ref="Q54:R54"/>
-    <mergeCell ref="Q55:R55"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="Q59:R59"/>
+    <mergeCell ref="Q60:R60"/>
     <mergeCell ref="Q25:R25"/>
     <mergeCell ref="Q26:R26"/>
     <mergeCell ref="Q27:R27"/>
@@ -2465,7 +2564,7 @@
     <mergeCell ref="Q34:R34"/>
     <mergeCell ref="Q35:R35"/>
     <mergeCell ref="Q36:R36"/>
-    <mergeCell ref="Q53:R53"/>
+    <mergeCell ref="Q58:R58"/>
     <mergeCell ref="Q20:R20"/>
     <mergeCell ref="Q21:R21"/>
     <mergeCell ref="Q22:R22"/>
@@ -2475,14 +2574,14 @@
     <mergeCell ref="Q16:R16"/>
     <mergeCell ref="Q18:R18"/>
     <mergeCell ref="Q19:R19"/>
-    <mergeCell ref="J55:K55"/>
+    <mergeCell ref="J60:K60"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="I1:L1"/>
     <mergeCell ref="J26:K26"/>
     <mergeCell ref="J27:K27"/>
     <mergeCell ref="J28:K28"/>
     <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J54:K54"/>
+    <mergeCell ref="J59:K59"/>
     <mergeCell ref="J21:K21"/>
     <mergeCell ref="J22:K22"/>
     <mergeCell ref="J23:K23"/>
@@ -2496,7 +2595,7 @@
     <mergeCell ref="J11:K11"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B58:C58"/>
     <mergeCell ref="J30:K30"/>
     <mergeCell ref="J31:K31"/>
     <mergeCell ref="J13:K13"/>
@@ -2546,14 +2645,14 @@
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="B59:C59"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B54:C54"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B21:C21"/>

</xml_diff>

<commit_message>
feat: improve analysis process and system prompts
- Introduce new subagent system prompts for movement intelligence, causality, thesis, and narrative (02a-02d)
- Refine existing system prompts for risk analyzer and report generator
- Update local server and handler flows to support improved processing
- Enhance financial math calculations and add new models to analyzer
- Update generated test outputs and accounting data
- Remove unused CreditIQ_Template_EEFF.docx fixture
</commit_message>
<xml_diff>
--- a/llms_calls_accounting.xlsx
+++ b/llms_calls_accounting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\03_iastronauts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59EEA947-1DEC-4F3D-9856-0523DA9FE88A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFBACB6E-686A-459F-A5A1-98E38F68CC58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{59B62FDA-1497-4401-82EC-1B2F7D702BCC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="109">
   <si>
     <t>Consumo Tokens CreditIQ</t>
   </si>
@@ -351,6 +351,21 @@
   </si>
   <si>
     <t>2026-06-05:22:16</t>
+  </si>
+  <si>
+    <t>2026-06-06:09:16</t>
+  </si>
+  <si>
+    <t>2026-06-06:09:20</t>
+  </si>
+  <si>
+    <t>2026-06-06:09:22</t>
+  </si>
+  <si>
+    <t>2026-06-06:09:26</t>
+  </si>
+  <si>
+    <t>2026-06-06:09:28</t>
   </si>
 </sst>
 </file>
@@ -562,14 +577,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -577,11 +595,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -604,22 +628,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -972,125 +987,125 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="I1" s="27" t="s">
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="I1" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="P1" s="27" t="s">
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="P1" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="Q1" s="27"/>
-      <c r="R1" s="27"/>
-      <c r="S1" s="27"/>
+      <c r="Q1" s="16"/>
+      <c r="R1" s="16"/>
+      <c r="S1" s="16"/>
     </row>
     <row r="2" spans="1:20" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26"/>
-      <c r="I2" s="24" t="s">
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="19"/>
+      <c r="I2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="26"/>
-      <c r="P2" s="24" t="s">
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="19"/>
+      <c r="P2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="Q2" s="25"/>
-      <c r="R2" s="25"/>
-      <c r="S2" s="26"/>
+      <c r="Q2" s="18"/>
+      <c r="R2" s="18"/>
+      <c r="S2" s="19"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="17" t="s">
+      <c r="B3" s="21"/>
+      <c r="C3" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="18"/>
-      <c r="I3" s="17" t="s">
+      <c r="D3" s="21"/>
+      <c r="I3" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="18"/>
-      <c r="K3" s="17" t="s">
+      <c r="J3" s="21"/>
+      <c r="K3" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="18"/>
-      <c r="P3" s="17" t="s">
+      <c r="L3" s="21"/>
+      <c r="P3" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="Q3" s="18"/>
-      <c r="R3" s="17" t="s">
+      <c r="Q3" s="21"/>
+      <c r="R3" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="S3" s="18"/>
+      <c r="S3" s="21"/>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="20"/>
-      <c r="D4" s="21"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="24"/>
       <c r="I4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="19" t="s">
+      <c r="J4" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="20"/>
-      <c r="L4" s="21"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="24"/>
       <c r="P4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="Q4" s="19" t="s">
+      <c r="Q4" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="R4" s="20"/>
-      <c r="S4" s="21"/>
+      <c r="R4" s="23"/>
+      <c r="S4" s="24"/>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="23"/>
+      <c r="C5" s="26"/>
       <c r="D5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="22" t="s">
+      <c r="J5" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="K5" s="23"/>
+      <c r="K5" s="26"/>
       <c r="L5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="P5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="Q5" s="22" t="s">
+      <c r="Q5" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="R5" s="23"/>
+      <c r="R5" s="26"/>
       <c r="S5" s="4" t="s">
         <v>8</v>
       </c>
@@ -1099,10 +1114,10 @@
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="12"/>
+      <c r="C6" s="11"/>
       <c r="D6" s="2" t="s">
         <v>10</v>
       </c>
@@ -1112,10 +1127,10 @@
       <c r="I6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J6" s="11" t="s">
+      <c r="J6" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="K6" s="12"/>
+      <c r="K6" s="11"/>
       <c r="L6" s="2" t="s">
         <v>35</v>
       </c>
@@ -1125,10 +1140,10 @@
       <c r="P6" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="Q6" s="11" t="s">
+      <c r="Q6" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="R6" s="12"/>
+      <c r="R6" s="11"/>
       <c r="S6" s="2" t="s">
         <v>23</v>
       </c>
@@ -1140,10 +1155,10 @@
       <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="12"/>
+      <c r="C7" s="11"/>
       <c r="D7" s="2" t="s">
         <v>11</v>
       </c>
@@ -1153,10 +1168,10 @@
       <c r="I7" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="J7" s="11" t="s">
+      <c r="J7" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="K7" s="12"/>
+      <c r="K7" s="11"/>
       <c r="L7" s="2" t="s">
         <v>37</v>
       </c>
@@ -1166,10 +1181,10 @@
       <c r="P7" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="Q7" s="11" t="s">
+      <c r="Q7" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="R7" s="12"/>
+      <c r="R7" s="11"/>
       <c r="S7" s="2" t="s">
         <v>44</v>
       </c>
@@ -1181,10 +1196,10 @@
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="12"/>
+      <c r="C8" s="11"/>
       <c r="D8" s="2" t="s">
         <v>10</v>
       </c>
@@ -1194,10 +1209,10 @@
       <c r="I8" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="J8" s="11" t="s">
+      <c r="J8" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="K8" s="12"/>
+      <c r="K8" s="11"/>
       <c r="L8" s="2" t="s">
         <v>23</v>
       </c>
@@ -1207,10 +1222,10 @@
       <c r="P8" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="Q8" s="11" t="s">
+      <c r="Q8" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="R8" s="12"/>
+      <c r="R8" s="11"/>
       <c r="S8" s="2" t="s">
         <v>49</v>
       </c>
@@ -1222,10 +1237,10 @@
       <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="12"/>
+      <c r="C9" s="11"/>
       <c r="D9" s="2" t="s">
         <v>16</v>
       </c>
@@ -1235,10 +1250,10 @@
       <c r="I9" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="J9" s="11" t="s">
+      <c r="J9" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="K9" s="12"/>
+      <c r="K9" s="11"/>
       <c r="L9" s="2" t="s">
         <v>28</v>
       </c>
@@ -1248,10 +1263,10 @@
       <c r="P9" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="Q9" s="11" t="s">
+      <c r="Q9" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="R9" s="12"/>
+      <c r="R9" s="11"/>
       <c r="S9" s="2" t="s">
         <v>52</v>
       </c>
@@ -1263,10 +1278,10 @@
       <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="12"/>
+      <c r="C10" s="11"/>
       <c r="D10" s="2" t="s">
         <v>10</v>
       </c>
@@ -1276,10 +1291,10 @@
       <c r="I10" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="J10" s="11" t="s">
+      <c r="J10" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="K10" s="12"/>
+      <c r="K10" s="11"/>
       <c r="L10" s="2" t="s">
         <v>23</v>
       </c>
@@ -1289,10 +1304,10 @@
       <c r="P10" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="Q10" s="11" t="s">
+      <c r="Q10" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="R10" s="12"/>
+      <c r="R10" s="11"/>
       <c r="S10" s="2" t="s">
         <v>28</v>
       </c>
@@ -1304,10 +1319,10 @@
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="12"/>
+      <c r="C11" s="11"/>
       <c r="D11" s="2" t="s">
         <v>18</v>
       </c>
@@ -1317,10 +1332,10 @@
       <c r="I11" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="J11" s="11" t="s">
+      <c r="J11" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="K11" s="12"/>
+      <c r="K11" s="11"/>
       <c r="L11" s="2" t="s">
         <v>46</v>
       </c>
@@ -1330,10 +1345,10 @@
       <c r="P11" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="Q11" s="11" t="s">
+      <c r="Q11" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="R11" s="12"/>
+      <c r="R11" s="11"/>
       <c r="S11" s="2" t="s">
         <v>46</v>
       </c>
@@ -1345,10 +1360,10 @@
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="12"/>
+      <c r="C12" s="11"/>
       <c r="D12" s="2" t="s">
         <v>10</v>
       </c>
@@ -1371,10 +1386,10 @@
       <c r="P12" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="Q12" s="11" t="s">
+      <c r="Q12" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="R12" s="12"/>
+      <c r="R12" s="11"/>
       <c r="S12" s="2" t="s">
         <v>18</v>
       </c>
@@ -1386,10 +1401,10 @@
       <c r="A13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="12"/>
+      <c r="C13" s="11"/>
       <c r="D13" s="2" t="s">
         <v>22</v>
       </c>
@@ -1399,10 +1414,10 @@
       <c r="I13" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="J13" s="11" t="s">
+      <c r="J13" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="K13" s="12"/>
+      <c r="K13" s="11"/>
       <c r="L13" s="2" t="s">
         <v>23</v>
       </c>
@@ -1412,10 +1427,10 @@
       <c r="P13" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="Q13" s="11" t="s">
+      <c r="Q13" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="R13" s="12"/>
+      <c r="R13" s="11"/>
       <c r="S13" s="2" t="s">
         <v>11</v>
       </c>
@@ -1427,10 +1442,10 @@
       <c r="A14" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="16"/>
+      <c r="C14" s="28"/>
       <c r="D14" s="7" t="s">
         <v>23</v>
       </c>
@@ -1444,10 +1459,10 @@
       <c r="I14" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="J14" s="11" t="s">
+      <c r="J14" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="K14" s="12"/>
+      <c r="K14" s="11"/>
       <c r="L14" s="2" t="s">
         <v>49</v>
       </c>
@@ -1457,10 +1472,10 @@
       <c r="P14" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="Q14" s="11" t="s">
+      <c r="Q14" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="R14" s="12"/>
+      <c r="R14" s="11"/>
       <c r="S14" s="2" t="s">
         <v>11</v>
       </c>
@@ -1472,10 +1487,10 @@
       <c r="A15" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="12"/>
+      <c r="C15" s="11"/>
       <c r="D15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1485,10 +1500,10 @@
       <c r="I15" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="J15" s="11" t="s">
+      <c r="J15" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="K15" s="12"/>
+      <c r="K15" s="11"/>
       <c r="L15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1498,10 +1513,10 @@
       <c r="P15" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="Q15" s="11" t="s">
+      <c r="Q15" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="R15" s="12"/>
+      <c r="R15" s="11"/>
       <c r="S15" s="2" t="s">
         <v>11</v>
       </c>
@@ -1513,10 +1528,10 @@
       <c r="A16" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="12"/>
+      <c r="C16" s="11"/>
       <c r="D16" s="2" t="s">
         <v>23</v>
       </c>
@@ -1526,10 +1541,10 @@
       <c r="I16" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="J16" s="11" t="s">
+      <c r="J16" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="K16" s="12"/>
+      <c r="K16" s="11"/>
       <c r="L16" s="2" t="s">
         <v>10</v>
       </c>
@@ -1539,10 +1554,10 @@
       <c r="P16" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="Q16" s="11" t="s">
+      <c r="Q16" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="R16" s="12"/>
+      <c r="R16" s="11"/>
       <c r="S16" s="2" t="s">
         <v>23</v>
       </c>
@@ -1554,10 +1569,10 @@
       <c r="A17" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C17" s="12"/>
+      <c r="C17" s="11"/>
       <c r="D17" s="2" t="s">
         <v>28</v>
       </c>
@@ -1565,8 +1580,8 @@
         <v>42</v>
       </c>
       <c r="I17" s="2"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="12"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="11"/>
       <c r="L17" s="2"/>
       <c r="P17" s="2" t="s">
         <v>85</v>
@@ -1586,10 +1601,10 @@
       <c r="A18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="12"/>
+      <c r="C18" s="11"/>
       <c r="D18" s="2" t="s">
         <v>23</v>
       </c>
@@ -1597,16 +1612,16 @@
         <v>42</v>
       </c>
       <c r="I18" s="2"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="12"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="11"/>
       <c r="L18" s="2"/>
       <c r="P18" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="Q18" s="11" t="s">
+      <c r="Q18" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="R18" s="12"/>
+      <c r="R18" s="11"/>
       <c r="S18" s="2" t="s">
         <v>23</v>
       </c>
@@ -1618,10 +1633,10 @@
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="12"/>
+      <c r="C19" s="11"/>
       <c r="D19" s="2" t="s">
         <v>28</v>
       </c>
@@ -1629,16 +1644,16 @@
         <v>42</v>
       </c>
       <c r="I19" s="2"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="12"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="11"/>
       <c r="L19" s="2"/>
       <c r="P19" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="Q19" s="11" t="s">
+      <c r="Q19" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="R19" s="12"/>
+      <c r="R19" s="11"/>
       <c r="S19" s="2" t="s">
         <v>49</v>
       </c>
@@ -1650,10 +1665,10 @@
       <c r="A20" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C20" s="12"/>
+      <c r="C20" s="11"/>
       <c r="D20" s="2" t="s">
         <v>35</v>
       </c>
@@ -1661,16 +1676,16 @@
         <v>42</v>
       </c>
       <c r="I20" s="2"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="12"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="11"/>
       <c r="L20" s="2"/>
       <c r="P20" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="Q20" s="11" t="s">
+      <c r="Q20" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="R20" s="12"/>
+      <c r="R20" s="11"/>
       <c r="S20" s="2" t="s">
         <v>23</v>
       </c>
@@ -1682,10 +1697,10 @@
       <c r="A21" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C21" s="12"/>
+      <c r="C21" s="11"/>
       <c r="D21" s="2" t="s">
         <v>28</v>
       </c>
@@ -1693,16 +1708,16 @@
         <v>42</v>
       </c>
       <c r="I21" s="2"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="12"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="11"/>
       <c r="L21" s="2"/>
       <c r="P21" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="Q21" s="11" t="s">
+      <c r="Q21" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="R21" s="12"/>
+      <c r="R21" s="11"/>
       <c r="S21" s="2" t="s">
         <v>46</v>
       </c>
@@ -1714,10 +1729,10 @@
       <c r="A22" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="12"/>
+      <c r="C22" s="11"/>
       <c r="D22" s="2" t="s">
         <v>28</v>
       </c>
@@ -1725,22 +1740,22 @@
         <v>42</v>
       </c>
       <c r="I22" s="2"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="12"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="11"/>
       <c r="L22" s="2"/>
       <c r="P22" s="2"/>
-      <c r="Q22" s="11"/>
-      <c r="R22" s="12"/>
+      <c r="Q22" s="10"/>
+      <c r="R22" s="11"/>
       <c r="S22" s="2"/>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C23" s="12"/>
+      <c r="C23" s="11"/>
       <c r="D23" s="2" t="s">
         <v>44</v>
       </c>
@@ -1748,22 +1763,22 @@
         <v>42</v>
       </c>
       <c r="I23" s="2"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="12"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="11"/>
       <c r="L23" s="2"/>
       <c r="P23" s="2"/>
-      <c r="Q23" s="11"/>
-      <c r="R23" s="12"/>
+      <c r="Q23" s="10"/>
+      <c r="R23" s="11"/>
       <c r="S23" s="2"/>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C24" s="12"/>
+      <c r="C24" s="11"/>
       <c r="D24" s="2" t="s">
         <v>28</v>
       </c>
@@ -1771,22 +1786,22 @@
         <v>42</v>
       </c>
       <c r="I24" s="2"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="12"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="11"/>
       <c r="L24" s="2"/>
       <c r="P24" s="2"/>
-      <c r="Q24" s="11"/>
-      <c r="R24" s="12"/>
+      <c r="Q24" s="10"/>
+      <c r="R24" s="11"/>
       <c r="S24" s="2"/>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="C25" s="12"/>
+      <c r="C25" s="11"/>
       <c r="D25" s="2" t="s">
         <v>46</v>
       </c>
@@ -1794,22 +1809,22 @@
         <v>42</v>
       </c>
       <c r="I25" s="2"/>
-      <c r="J25" s="11"/>
-      <c r="K25" s="12"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="11"/>
       <c r="L25" s="2"/>
       <c r="P25" s="2"/>
-      <c r="Q25" s="11"/>
-      <c r="R25" s="12"/>
+      <c r="Q25" s="10"/>
+      <c r="R25" s="11"/>
       <c r="S25" s="2"/>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C26" s="12"/>
+      <c r="C26" s="11"/>
       <c r="D26" s="2" t="s">
         <v>11</v>
       </c>
@@ -1817,22 +1832,22 @@
         <v>42</v>
       </c>
       <c r="I26" s="2"/>
-      <c r="J26" s="11"/>
-      <c r="K26" s="12"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="11"/>
       <c r="L26" s="2"/>
       <c r="P26" s="2"/>
-      <c r="Q26" s="11"/>
-      <c r="R26" s="12"/>
+      <c r="Q26" s="10"/>
+      <c r="R26" s="11"/>
       <c r="S26" s="2"/>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C27" s="12"/>
+      <c r="C27" s="11"/>
       <c r="D27" s="2" t="s">
         <v>28</v>
       </c>
@@ -1840,22 +1855,22 @@
         <v>42</v>
       </c>
       <c r="I27" s="2"/>
-      <c r="J27" s="11"/>
-      <c r="K27" s="12"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="11"/>
       <c r="L27" s="2"/>
       <c r="P27" s="2"/>
-      <c r="Q27" s="11"/>
-      <c r="R27" s="12"/>
+      <c r="Q27" s="10"/>
+      <c r="R27" s="11"/>
       <c r="S27" s="2"/>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C28" s="12"/>
+      <c r="C28" s="11"/>
       <c r="D28" s="2" t="s">
         <v>28</v>
       </c>
@@ -1863,22 +1878,22 @@
         <v>42</v>
       </c>
       <c r="I28" s="2"/>
-      <c r="J28" s="11"/>
-      <c r="K28" s="12"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="11"/>
       <c r="L28" s="2"/>
       <c r="P28" s="2"/>
-      <c r="Q28" s="11"/>
-      <c r="R28" s="12"/>
+      <c r="Q28" s="10"/>
+      <c r="R28" s="11"/>
       <c r="S28" s="2"/>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B29" s="11" t="s">
+      <c r="B29" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="C29" s="12"/>
+      <c r="C29" s="11"/>
       <c r="D29" s="2" t="s">
         <v>46</v>
       </c>
@@ -1886,22 +1901,22 @@
         <v>42</v>
       </c>
       <c r="I29" s="2"/>
-      <c r="J29" s="11"/>
-      <c r="K29" s="12"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="11"/>
       <c r="L29" s="2"/>
       <c r="P29" s="2"/>
-      <c r="Q29" s="11"/>
-      <c r="R29" s="12"/>
+      <c r="Q29" s="10"/>
+      <c r="R29" s="11"/>
       <c r="S29" s="2"/>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C30" s="12"/>
+      <c r="C30" s="11"/>
       <c r="D30" s="2" t="s">
         <v>28</v>
       </c>
@@ -1909,22 +1924,22 @@
         <v>42</v>
       </c>
       <c r="I30" s="2"/>
-      <c r="J30" s="11"/>
-      <c r="K30" s="12"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="11"/>
       <c r="L30" s="2"/>
       <c r="P30" s="2"/>
-      <c r="Q30" s="11"/>
-      <c r="R30" s="12"/>
+      <c r="Q30" s="10"/>
+      <c r="R30" s="11"/>
       <c r="S30" s="2"/>
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C31" s="12"/>
+      <c r="C31" s="11"/>
       <c r="D31" s="2" t="s">
         <v>23</v>
       </c>
@@ -1932,22 +1947,22 @@
         <v>42</v>
       </c>
       <c r="I31" s="2"/>
-      <c r="J31" s="11"/>
-      <c r="K31" s="12"/>
+      <c r="J31" s="10"/>
+      <c r="K31" s="11"/>
       <c r="L31" s="2"/>
       <c r="P31" s="2"/>
-      <c r="Q31" s="11"/>
-      <c r="R31" s="12"/>
+      <c r="Q31" s="10"/>
+      <c r="R31" s="11"/>
       <c r="S31" s="2"/>
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C32" s="12"/>
+      <c r="C32" s="11"/>
       <c r="D32" s="2" t="s">
         <v>23</v>
       </c>
@@ -1955,22 +1970,22 @@
         <v>42</v>
       </c>
       <c r="I32" s="2"/>
-      <c r="J32" s="11"/>
-      <c r="K32" s="12"/>
+      <c r="J32" s="10"/>
+      <c r="K32" s="11"/>
       <c r="L32" s="2"/>
       <c r="P32" s="2"/>
-      <c r="Q32" s="11"/>
-      <c r="R32" s="12"/>
+      <c r="Q32" s="10"/>
+      <c r="R32" s="11"/>
       <c r="S32" s="2"/>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B33" s="11" t="s">
+      <c r="B33" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C33" s="12"/>
+      <c r="C33" s="11"/>
       <c r="D33" s="2" t="s">
         <v>23</v>
       </c>
@@ -1978,22 +1993,22 @@
         <v>42</v>
       </c>
       <c r="I33" s="2"/>
-      <c r="J33" s="11"/>
-      <c r="K33" s="12"/>
+      <c r="J33" s="10"/>
+      <c r="K33" s="11"/>
       <c r="L33" s="2"/>
       <c r="P33" s="2"/>
-      <c r="Q33" s="11"/>
-      <c r="R33" s="12"/>
+      <c r="Q33" s="10"/>
+      <c r="R33" s="11"/>
       <c r="S33" s="2"/>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B34" s="11" t="s">
+      <c r="B34" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C34" s="12"/>
+      <c r="C34" s="11"/>
       <c r="D34" s="2" t="s">
         <v>23</v>
       </c>
@@ -2001,22 +2016,22 @@
         <v>42</v>
       </c>
       <c r="I34" s="2"/>
-      <c r="J34" s="11"/>
-      <c r="K34" s="12"/>
+      <c r="J34" s="10"/>
+      <c r="K34" s="11"/>
       <c r="L34" s="2"/>
       <c r="P34" s="2"/>
-      <c r="Q34" s="11"/>
-      <c r="R34" s="12"/>
+      <c r="Q34" s="10"/>
+      <c r="R34" s="11"/>
       <c r="S34" s="2"/>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B35" s="11" t="s">
+      <c r="B35" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="C35" s="12"/>
+      <c r="C35" s="11"/>
       <c r="D35" s="2" t="s">
         <v>46</v>
       </c>
@@ -2024,22 +2039,22 @@
         <v>42</v>
       </c>
       <c r="I35" s="2"/>
-      <c r="J35" s="11"/>
-      <c r="K35" s="12"/>
+      <c r="J35" s="10"/>
+      <c r="K35" s="11"/>
       <c r="L35" s="2"/>
       <c r="P35" s="2"/>
-      <c r="Q35" s="11"/>
-      <c r="R35" s="12"/>
+      <c r="Q35" s="10"/>
+      <c r="R35" s="11"/>
       <c r="S35" s="2"/>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B36" s="11" t="s">
+      <c r="B36" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C36" s="12"/>
+      <c r="C36" s="11"/>
       <c r="D36" s="2" t="s">
         <v>89</v>
       </c>
@@ -2047,22 +2062,22 @@
         <v>42</v>
       </c>
       <c r="I36" s="2"/>
-      <c r="J36" s="11"/>
-      <c r="K36" s="12"/>
+      <c r="J36" s="10"/>
+      <c r="K36" s="11"/>
       <c r="L36" s="2"/>
       <c r="P36" s="2"/>
-      <c r="Q36" s="11"/>
-      <c r="R36" s="12"/>
+      <c r="Q36" s="10"/>
+      <c r="R36" s="11"/>
       <c r="S36" s="2"/>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B37" s="11" t="s">
+      <c r="B37" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C37" s="12"/>
+      <c r="C37" s="11"/>
       <c r="D37" s="2" t="s">
         <v>23</v>
       </c>
@@ -2082,10 +2097,10 @@
       <c r="A38" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B38" s="11" t="s">
+      <c r="B38" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="C38" s="12"/>
+      <c r="C38" s="11"/>
       <c r="D38" s="2" t="s">
         <v>46</v>
       </c>
@@ -2105,10 +2120,10 @@
       <c r="A39" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B39" s="11" t="s">
+      <c r="B39" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C39" s="12"/>
+      <c r="C39" s="11"/>
       <c r="D39" s="2" t="s">
         <v>11</v>
       </c>
@@ -2128,10 +2143,10 @@
       <c r="A40" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="C40" s="12"/>
+      <c r="C40" s="11"/>
       <c r="D40" s="2" t="s">
         <v>46</v>
       </c>
@@ -2151,10 +2166,10 @@
       <c r="A41" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="11" t="s">
+      <c r="B41" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C41" s="12"/>
+      <c r="C41" s="11"/>
       <c r="D41" s="2" t="s">
         <v>44</v>
       </c>
@@ -2174,10 +2189,10 @@
       <c r="A42" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B42" s="11" t="s">
+      <c r="B42" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C42" s="12"/>
+      <c r="C42" s="11"/>
       <c r="D42" s="2" t="s">
         <v>11</v>
       </c>
@@ -2197,10 +2212,10 @@
       <c r="A43" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B43" s="11" t="s">
+      <c r="B43" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="C43" s="12"/>
+      <c r="C43" s="11"/>
       <c r="D43" s="2" t="s">
         <v>46</v>
       </c>
@@ -2220,10 +2235,10 @@
       <c r="A44" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B44" s="11" t="s">
+      <c r="B44" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C44" s="12"/>
+      <c r="C44" s="11"/>
       <c r="D44" s="2" t="s">
         <v>44</v>
       </c>
@@ -2243,10 +2258,10 @@
       <c r="A45" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B45" s="11" t="s">
+      <c r="B45" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C45" s="12"/>
+      <c r="C45" s="11"/>
       <c r="D45" s="2" t="s">
         <v>23</v>
       </c>
@@ -2266,10 +2281,10 @@
       <c r="A46" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B46" s="11" t="s">
+      <c r="B46" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="C46" s="12"/>
+      <c r="C46" s="11"/>
       <c r="D46" s="2" t="s">
         <v>49</v>
       </c>
@@ -2289,10 +2304,10 @@
       <c r="A47" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B47" s="11" t="s">
+      <c r="B47" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C47" s="12"/>
+      <c r="C47" s="11"/>
       <c r="D47" s="2" t="s">
         <v>23</v>
       </c>
@@ -2312,10 +2327,10 @@
       <c r="A48" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B48" s="11" t="s">
+      <c r="B48" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C48" s="12"/>
+      <c r="C48" s="11"/>
       <c r="D48" s="2" t="s">
         <v>28</v>
       </c>
@@ -2335,10 +2350,10 @@
       <c r="A49" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B49" s="11" t="s">
+      <c r="B49" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C49" s="12"/>
+      <c r="C49" s="11"/>
       <c r="D49" s="2" t="s">
         <v>23</v>
       </c>
@@ -2355,10 +2370,19 @@
       <c r="S49" s="2"/>
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A50" s="2"/>
-      <c r="B50" s="28"/>
-      <c r="C50" s="29"/>
-      <c r="D50" s="2"/>
+      <c r="A50" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B50" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C50" s="11"/>
+      <c r="D50" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E50" t="s">
+        <v>42</v>
+      </c>
       <c r="I50" s="2"/>
       <c r="J50" s="8"/>
       <c r="K50" s="9"/>
@@ -2369,10 +2393,19 @@
       <c r="S50" s="2"/>
     </row>
     <row r="51" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A51" s="2"/>
-      <c r="B51" s="28"/>
-      <c r="C51" s="29"/>
-      <c r="D51" s="2"/>
+      <c r="A51" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B51" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C51" s="11"/>
+      <c r="D51" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E51" t="s">
+        <v>42</v>
+      </c>
       <c r="I51" s="2"/>
       <c r="J51" s="8"/>
       <c r="K51" s="9"/>
@@ -2383,10 +2416,19 @@
       <c r="S51" s="2"/>
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A52" s="2"/>
-      <c r="B52" s="28"/>
-      <c r="C52" s="29"/>
-      <c r="D52" s="2"/>
+      <c r="A52" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B52" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C52" s="11"/>
+      <c r="D52" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E52" t="s">
+        <v>42</v>
+      </c>
       <c r="I52" s="2"/>
       <c r="J52" s="8"/>
       <c r="K52" s="9"/>
@@ -2397,10 +2439,19 @@
       <c r="S52" s="2"/>
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A53" s="2"/>
-      <c r="B53" s="28"/>
-      <c r="C53" s="29"/>
-      <c r="D53" s="2"/>
+      <c r="A53" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B53" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C53" s="11"/>
+      <c r="D53" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53" t="s">
+        <v>42</v>
+      </c>
       <c r="I53" s="2"/>
       <c r="J53" s="8"/>
       <c r="K53" s="9"/>
@@ -2411,10 +2462,19 @@
       <c r="S53" s="2"/>
     </row>
     <row r="54" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A54" s="2"/>
-      <c r="B54" s="28"/>
-      <c r="C54" s="29"/>
-      <c r="D54" s="2"/>
+      <c r="A54" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B54" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="C54" s="11"/>
+      <c r="D54" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E54" t="s">
+        <v>42</v>
+      </c>
       <c r="I54" s="2"/>
       <c r="J54" s="8"/>
       <c r="K54" s="9"/>
@@ -2426,8 +2486,8 @@
     </row>
     <row r="55" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A55" s="2"/>
-      <c r="B55" s="28"/>
-      <c r="C55" s="29"/>
+      <c r="B55" s="12"/>
+      <c r="C55" s="13"/>
       <c r="D55" s="2"/>
       <c r="I55" s="2"/>
       <c r="J55" s="8"/>
@@ -2440,8 +2500,8 @@
     </row>
     <row r="56" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="2"/>
-      <c r="B56" s="28"/>
-      <c r="C56" s="29"/>
+      <c r="B56" s="12"/>
+      <c r="C56" s="13"/>
       <c r="D56" s="2"/>
       <c r="I56" s="2"/>
       <c r="J56" s="8"/>
@@ -2454,8 +2514,8 @@
     </row>
     <row r="57" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A57" s="2"/>
-      <c r="B57" s="28"/>
-      <c r="C57" s="29"/>
+      <c r="B57" s="12"/>
+      <c r="C57" s="13"/>
       <c r="D57" s="2"/>
       <c r="I57" s="2"/>
       <c r="J57" s="8"/>
@@ -2468,64 +2528,183 @@
     </row>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A58" s="2"/>
-      <c r="B58" s="28"/>
-      <c r="C58" s="29"/>
+      <c r="B58" s="12"/>
+      <c r="C58" s="13"/>
       <c r="D58" s="2"/>
       <c r="I58" s="2"/>
-      <c r="J58" s="11"/>
-      <c r="K58" s="12"/>
+      <c r="J58" s="10"/>
+      <c r="K58" s="11"/>
       <c r="L58" s="2"/>
       <c r="P58" s="2"/>
-      <c r="Q58" s="11"/>
-      <c r="R58" s="12"/>
+      <c r="Q58" s="10"/>
+      <c r="R58" s="11"/>
       <c r="S58" s="2"/>
     </row>
     <row r="59" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A59" s="2"/>
-      <c r="B59" s="11"/>
-      <c r="C59" s="12"/>
+      <c r="B59" s="10"/>
+      <c r="C59" s="11"/>
       <c r="D59" s="2"/>
       <c r="I59" s="2"/>
-      <c r="J59" s="11"/>
-      <c r="K59" s="12"/>
+      <c r="J59" s="10"/>
+      <c r="K59" s="11"/>
       <c r="L59" s="2"/>
       <c r="P59" s="2"/>
-      <c r="Q59" s="11"/>
-      <c r="R59" s="12"/>
+      <c r="Q59" s="10"/>
+      <c r="R59" s="11"/>
       <c r="S59" s="2"/>
     </row>
     <row r="60" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A60" s="3"/>
-      <c r="B60" s="13"/>
-      <c r="C60" s="14"/>
+      <c r="B60" s="14"/>
+      <c r="C60" s="15"/>
       <c r="D60" s="3"/>
       <c r="I60" s="3"/>
-      <c r="J60" s="13"/>
-      <c r="K60" s="14"/>
+      <c r="J60" s="14"/>
+      <c r="K60" s="15"/>
       <c r="L60" s="3"/>
       <c r="P60" s="3"/>
-      <c r="Q60" s="13"/>
-      <c r="R60" s="14"/>
+      <c r="Q60" s="14"/>
+      <c r="R60" s="15"/>
       <c r="S60" s="3"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="10"/>
-      <c r="C61" s="10"/>
+      <c r="B61" s="29"/>
+      <c r="C61" s="29"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B62" s="10"/>
-      <c r="C62" s="10"/>
+      <c r="B62" s="29"/>
+      <c r="C62" s="29"/>
     </row>
     <row r="63" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B63" s="10"/>
-      <c r="C63" s="10"/>
+      <c r="B63" s="29"/>
+      <c r="C63" s="29"/>
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B64" s="10"/>
-      <c r="C64" s="10"/>
+      <c r="B64" s="29"/>
+      <c r="C64" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="143">
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="P1:S1"/>
+    <mergeCell ref="P2:S2"/>
+    <mergeCell ref="P3:Q3"/>
+    <mergeCell ref="R3:S3"/>
+    <mergeCell ref="Q4:S4"/>
+    <mergeCell ref="Q10:R10"/>
+    <mergeCell ref="Q11:R11"/>
+    <mergeCell ref="Q12:R12"/>
+    <mergeCell ref="Q13:R13"/>
+    <mergeCell ref="Q14:R14"/>
+    <mergeCell ref="Q5:R5"/>
+    <mergeCell ref="Q6:R6"/>
+    <mergeCell ref="Q7:R7"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="Q9:R9"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="J60:K60"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="I1:L1"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J59:K59"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="Q20:R20"/>
+    <mergeCell ref="Q21:R21"/>
+    <mergeCell ref="Q22:R22"/>
+    <mergeCell ref="Q23:R23"/>
+    <mergeCell ref="Q24:R24"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="Q16:R16"/>
+    <mergeCell ref="Q18:R18"/>
+    <mergeCell ref="Q19:R19"/>
+    <mergeCell ref="Q59:R59"/>
+    <mergeCell ref="Q60:R60"/>
+    <mergeCell ref="Q25:R25"/>
+    <mergeCell ref="Q26:R26"/>
+    <mergeCell ref="Q27:R27"/>
+    <mergeCell ref="Q28:R28"/>
+    <mergeCell ref="Q29:R29"/>
+    <mergeCell ref="Q30:R30"/>
+    <mergeCell ref="Q31:R31"/>
+    <mergeCell ref="Q32:R32"/>
+    <mergeCell ref="Q33:R33"/>
+    <mergeCell ref="Q34:R34"/>
+    <mergeCell ref="Q35:R35"/>
+    <mergeCell ref="Q36:R36"/>
+    <mergeCell ref="Q58:R58"/>
     <mergeCell ref="J32:K32"/>
     <mergeCell ref="J33:K33"/>
     <mergeCell ref="J34:K34"/>
@@ -2550,125 +2729,6 @@
     <mergeCell ref="B51:C51"/>
     <mergeCell ref="B52:C52"/>
     <mergeCell ref="B53:C53"/>
-    <mergeCell ref="Q59:R59"/>
-    <mergeCell ref="Q60:R60"/>
-    <mergeCell ref="Q25:R25"/>
-    <mergeCell ref="Q26:R26"/>
-    <mergeCell ref="Q27:R27"/>
-    <mergeCell ref="Q28:R28"/>
-    <mergeCell ref="Q29:R29"/>
-    <mergeCell ref="Q30:R30"/>
-    <mergeCell ref="Q31:R31"/>
-    <mergeCell ref="Q32:R32"/>
-    <mergeCell ref="Q33:R33"/>
-    <mergeCell ref="Q34:R34"/>
-    <mergeCell ref="Q35:R35"/>
-    <mergeCell ref="Q36:R36"/>
-    <mergeCell ref="Q58:R58"/>
-    <mergeCell ref="Q20:R20"/>
-    <mergeCell ref="Q21:R21"/>
-    <mergeCell ref="Q22:R22"/>
-    <mergeCell ref="Q23:R23"/>
-    <mergeCell ref="Q24:R24"/>
-    <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="Q16:R16"/>
-    <mergeCell ref="Q18:R18"/>
-    <mergeCell ref="Q19:R19"/>
-    <mergeCell ref="J60:K60"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="I1:L1"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J59:K59"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="P1:S1"/>
-    <mergeCell ref="P2:S2"/>
-    <mergeCell ref="P3:Q3"/>
-    <mergeCell ref="R3:S3"/>
-    <mergeCell ref="Q4:S4"/>
-    <mergeCell ref="Q10:R10"/>
-    <mergeCell ref="Q11:R11"/>
-    <mergeCell ref="Q12:R12"/>
-    <mergeCell ref="Q13:R13"/>
-    <mergeCell ref="Q14:R14"/>
-    <mergeCell ref="Q5:R5"/>
-    <mergeCell ref="Q6:R6"/>
-    <mergeCell ref="Q7:R7"/>
-    <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="Q9:R9"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B59:C59"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B41:C41"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: Implement multi-agent routing and specialized role profiles
- Added  and  to establish specialized agent instructions and dynamic context management.
- Implemented  for inter-agent communication and state transition.
- Updated agent handlers (, , , , ) to utilize the new role profiles and handoff logic.
- Refactored shared models to align with the updated architecture.
- Added  in the frontend for mapping data keys to human-readable labels.
- Updated frontend components (, , ) and  to handle the new multi-agent API structure.
- Simplified  by removing market risk/stress scenario sections and renumbering the document.
- Updated architecture documentation ( and ) to reflect the new agent interactions.
</commit_message>
<xml_diff>
--- a/llms_calls_accounting.xlsx
+++ b/llms_calls_accounting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\03_iastronauts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFBACB6E-686A-459F-A5A1-98E38F68CC58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8DEB14D-38E2-4C36-A80F-1C3D03DA33A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{59B62FDA-1497-4401-82EC-1B2F7D702BCC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="121">
   <si>
     <t>Consumo Tokens CreditIQ</t>
   </si>
@@ -366,6 +366,42 @@
   </si>
   <si>
     <t>2026-06-06:09:28</t>
+  </si>
+  <si>
+    <t>2026-06-09:09:10</t>
+  </si>
+  <si>
+    <t>2026-06-09:09:13</t>
+  </si>
+  <si>
+    <t>2026-06-09:09:16</t>
+  </si>
+  <si>
+    <t>2026-06-09:21:48</t>
+  </si>
+  <si>
+    <t>2026-06-09:21:52</t>
+  </si>
+  <si>
+    <t>2026-06-09:21:53</t>
+  </si>
+  <si>
+    <t>2026-06-09:21:55</t>
+  </si>
+  <si>
+    <t>2026-06-09:22:40</t>
+  </si>
+  <si>
+    <t>2026-06-09:22:48</t>
+  </si>
+  <si>
+    <t>2026-06-09:22:49</t>
+  </si>
+  <si>
+    <t>2026-06-09:22:51</t>
+  </si>
+  <si>
+    <t>2026-06-09:23:01</t>
   </si>
 </sst>
 </file>
@@ -560,7 +596,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
@@ -582,12 +618,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -971,7 +1001,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B052F0D6-0E50-4E03-8DA0-D70F625DE32B}">
-  <dimension ref="A1:T64"/>
+  <dimension ref="A1:T71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.85546875" customWidth="1"/>
@@ -987,125 +1017,125 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="I1" s="16" t="s">
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="I1" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="P1" s="16" t="s">
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="P1" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="Q1" s="16"/>
-      <c r="R1" s="16"/>
-      <c r="S1" s="16"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
     </row>
     <row r="2" spans="1:20" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="19"/>
-      <c r="I2" s="17" t="s">
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="17"/>
+      <c r="I2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="19"/>
-      <c r="P2" s="17" t="s">
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="17"/>
+      <c r="P2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="Q2" s="18"/>
-      <c r="R2" s="18"/>
-      <c r="S2" s="19"/>
+      <c r="Q2" s="16"/>
+      <c r="R2" s="16"/>
+      <c r="S2" s="17"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="21"/>
-      <c r="C3" s="20" t="s">
+      <c r="B3" s="19"/>
+      <c r="C3" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="21"/>
-      <c r="I3" s="20" t="s">
+      <c r="D3" s="19"/>
+      <c r="I3" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="21"/>
-      <c r="K3" s="20" t="s">
+      <c r="J3" s="19"/>
+      <c r="K3" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="21"/>
-      <c r="P3" s="20" t="s">
+      <c r="L3" s="19"/>
+      <c r="P3" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="Q3" s="21"/>
-      <c r="R3" s="20" t="s">
+      <c r="Q3" s="19"/>
+      <c r="R3" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="S3" s="21"/>
+      <c r="S3" s="19"/>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="24"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="22"/>
       <c r="I4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="22" t="s">
+      <c r="J4" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="23"/>
-      <c r="L4" s="24"/>
+      <c r="K4" s="21"/>
+      <c r="L4" s="22"/>
       <c r="P4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="Q4" s="22" t="s">
+      <c r="Q4" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="R4" s="23"/>
-      <c r="S4" s="24"/>
+      <c r="R4" s="21"/>
+      <c r="S4" s="22"/>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="26"/>
+      <c r="C5" s="24"/>
       <c r="D5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="25" t="s">
+      <c r="J5" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="K5" s="26"/>
+      <c r="K5" s="24"/>
       <c r="L5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="P5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="Q5" s="25" t="s">
+      <c r="Q5" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="R5" s="26"/>
+      <c r="R5" s="24"/>
       <c r="S5" s="4" t="s">
         <v>8</v>
       </c>
@@ -1442,10 +1472,10 @@
       <c r="A14" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="28"/>
+      <c r="C14" s="26"/>
       <c r="D14" s="7" t="s">
         <v>23</v>
       </c>
@@ -2485,10 +2515,19 @@
       <c r="S54" s="2"/>
     </row>
     <row r="55" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A55" s="2"/>
-      <c r="B55" s="12"/>
-      <c r="C55" s="13"/>
-      <c r="D55" s="2"/>
+      <c r="A55" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B55" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C55" s="11"/>
+      <c r="D55" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E55" t="s">
+        <v>42</v>
+      </c>
       <c r="I55" s="2"/>
       <c r="J55" s="8"/>
       <c r="K55" s="9"/>
@@ -2499,10 +2538,19 @@
       <c r="S55" s="2"/>
     </row>
     <row r="56" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A56" s="2"/>
-      <c r="B56" s="12"/>
-      <c r="C56" s="13"/>
-      <c r="D56" s="2"/>
+      <c r="A56" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B56" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C56" s="11"/>
+      <c r="D56" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E56" t="s">
+        <v>42</v>
+      </c>
       <c r="I56" s="2"/>
       <c r="J56" s="8"/>
       <c r="K56" s="9"/>
@@ -2513,10 +2561,19 @@
       <c r="S56" s="2"/>
     </row>
     <row r="57" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A57" s="2"/>
-      <c r="B57" s="12"/>
-      <c r="C57" s="13"/>
-      <c r="D57" s="2"/>
+      <c r="A57" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B57" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C57" s="11"/>
+      <c r="D57" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57" t="s">
+        <v>42</v>
+      </c>
       <c r="I57" s="2"/>
       <c r="J57" s="8"/>
       <c r="K57" s="9"/>
@@ -2527,10 +2584,19 @@
       <c r="S57" s="2"/>
     </row>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A58" s="2"/>
-      <c r="B58" s="12"/>
-      <c r="C58" s="13"/>
-      <c r="D58" s="2"/>
+      <c r="A58" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B58" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C58" s="11"/>
+      <c r="D58" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E58" t="s">
+        <v>42</v>
+      </c>
       <c r="I58" s="2"/>
       <c r="J58" s="10"/>
       <c r="K58" s="11"/>
@@ -2541,59 +2607,236 @@
       <c r="S58" s="2"/>
     </row>
     <row r="59" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A59" s="2"/>
-      <c r="B59" s="10"/>
+      <c r="A59" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B59" s="10" t="s">
+        <v>13</v>
+      </c>
       <c r="C59" s="11"/>
-      <c r="D59" s="2"/>
+      <c r="D59" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E59" t="s">
+        <v>42</v>
+      </c>
       <c r="I59" s="2"/>
-      <c r="J59" s="10"/>
-      <c r="K59" s="11"/>
+      <c r="J59" s="8"/>
+      <c r="K59" s="9"/>
       <c r="L59" s="2"/>
       <c r="P59" s="2"/>
-      <c r="Q59" s="10"/>
-      <c r="R59" s="11"/>
+      <c r="Q59" s="8"/>
+      <c r="R59" s="9"/>
       <c r="S59" s="2"/>
     </row>
     <row r="60" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A60" s="3"/>
-      <c r="B60" s="14"/>
-      <c r="C60" s="15"/>
-      <c r="D60" s="3"/>
-      <c r="I60" s="3"/>
-      <c r="J60" s="14"/>
-      <c r="K60" s="15"/>
-      <c r="L60" s="3"/>
-      <c r="P60" s="3"/>
-      <c r="Q60" s="14"/>
-      <c r="R60" s="15"/>
-      <c r="S60" s="3"/>
+      <c r="A60" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B60" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C60" s="11"/>
+      <c r="D60" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E60" t="s">
+        <v>42</v>
+      </c>
+      <c r="I60" s="2"/>
+      <c r="J60" s="8"/>
+      <c r="K60" s="9"/>
+      <c r="L60" s="2"/>
+      <c r="P60" s="2"/>
+      <c r="Q60" s="8"/>
+      <c r="R60" s="9"/>
+      <c r="S60" s="2"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="29"/>
-      <c r="C61" s="29"/>
+      <c r="A61" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B61" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C61" s="11"/>
+      <c r="D61" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E61" t="s">
+        <v>42</v>
+      </c>
+      <c r="I61" s="2"/>
+      <c r="J61" s="8"/>
+      <c r="K61" s="9"/>
+      <c r="L61" s="2"/>
+      <c r="P61" s="2"/>
+      <c r="Q61" s="8"/>
+      <c r="R61" s="9"/>
+      <c r="S61" s="2"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B62" s="29"/>
-      <c r="C62" s="29"/>
+      <c r="A62" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B62" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C62" s="11"/>
+      <c r="D62" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E62" t="s">
+        <v>42</v>
+      </c>
+      <c r="I62" s="2"/>
+      <c r="J62" s="8"/>
+      <c r="K62" s="9"/>
+      <c r="L62" s="2"/>
+      <c r="P62" s="2"/>
+      <c r="Q62" s="8"/>
+      <c r="R62" s="9"/>
+      <c r="S62" s="2"/>
     </row>
     <row r="63" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B63" s="29"/>
-      <c r="C63" s="29"/>
+      <c r="A63" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B63" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C63" s="11"/>
+      <c r="D63" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E63" t="s">
+        <v>42</v>
+      </c>
+      <c r="I63" s="2"/>
+      <c r="J63" s="8"/>
+      <c r="K63" s="9"/>
+      <c r="L63" s="2"/>
+      <c r="P63" s="2"/>
+      <c r="Q63" s="8"/>
+      <c r="R63" s="9"/>
+      <c r="S63" s="2"/>
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B64" s="29"/>
-      <c r="C64" s="29"/>
+      <c r="A64" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B64" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C64" s="11"/>
+      <c r="D64" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E64" t="s">
+        <v>42</v>
+      </c>
+      <c r="I64" s="2"/>
+      <c r="J64" s="8"/>
+      <c r="K64" s="9"/>
+      <c r="L64" s="2"/>
+      <c r="P64" s="2"/>
+      <c r="Q64" s="8"/>
+      <c r="R64" s="9"/>
+      <c r="S64" s="2"/>
+    </row>
+    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A65" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B65" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C65" s="11"/>
+      <c r="D65" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E65" t="s">
+        <v>42</v>
+      </c>
+      <c r="I65" s="2"/>
+      <c r="J65" s="8"/>
+      <c r="K65" s="9"/>
+      <c r="L65" s="2"/>
+      <c r="P65" s="2"/>
+      <c r="Q65" s="8"/>
+      <c r="R65" s="9"/>
+      <c r="S65" s="2"/>
+    </row>
+    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A66" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B66" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="C66" s="11"/>
+      <c r="D66" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E66" t="s">
+        <v>42</v>
+      </c>
+      <c r="I66" s="2"/>
+      <c r="J66" s="10"/>
+      <c r="K66" s="11"/>
+      <c r="L66" s="2"/>
+      <c r="P66" s="2"/>
+      <c r="Q66" s="10"/>
+      <c r="R66" s="11"/>
+      <c r="S66" s="2"/>
+    </row>
+    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A67" s="3"/>
+      <c r="B67" s="12"/>
+      <c r="C67" s="13"/>
+      <c r="D67" s="3"/>
+      <c r="I67" s="3"/>
+      <c r="J67" s="12"/>
+      <c r="K67" s="13"/>
+      <c r="L67" s="3"/>
+      <c r="P67" s="3"/>
+      <c r="Q67" s="12"/>
+      <c r="R67" s="13"/>
+      <c r="S67" s="3"/>
+    </row>
+    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B68" s="27"/>
+      <c r="C68" s="27"/>
+    </row>
+    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B69" s="27"/>
+      <c r="C69" s="27"/>
+    </row>
+    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B70" s="27"/>
+      <c r="C70" s="27"/>
+    </row>
+    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B71" s="27"/>
+      <c r="C71" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="143">
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="B18:C18"/>
+  <mergeCells count="150">
+    <mergeCell ref="B59:C59"/>
     <mergeCell ref="B60:C60"/>
     <mergeCell ref="B61:C61"/>
     <mergeCell ref="B62:C62"/>
     <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="B68:C68"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B70:C70"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="B66:C66"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B21:C21"/>
@@ -2657,14 +2900,14 @@
     <mergeCell ref="Q8:R8"/>
     <mergeCell ref="Q9:R9"/>
     <mergeCell ref="I2:L2"/>
-    <mergeCell ref="J60:K60"/>
+    <mergeCell ref="J67:K67"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="I1:L1"/>
     <mergeCell ref="J26:K26"/>
     <mergeCell ref="J27:K27"/>
     <mergeCell ref="J28:K28"/>
     <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J59:K59"/>
+    <mergeCell ref="J66:K66"/>
     <mergeCell ref="J21:K21"/>
     <mergeCell ref="J22:K22"/>
     <mergeCell ref="J23:K23"/>
@@ -2690,8 +2933,8 @@
     <mergeCell ref="Q16:R16"/>
     <mergeCell ref="Q18:R18"/>
     <mergeCell ref="Q19:R19"/>
-    <mergeCell ref="Q59:R59"/>
-    <mergeCell ref="Q60:R60"/>
+    <mergeCell ref="Q66:R66"/>
+    <mergeCell ref="Q67:R67"/>
     <mergeCell ref="Q25:R25"/>
     <mergeCell ref="Q26:R26"/>
     <mergeCell ref="Q27:R27"/>

</xml_diff>